<commit_message>
docs: update the HL7 and CCDA to FHIR conversion specification documents to add the Part2 related changes and Location resources
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" firstSheet="3" activeTab="7"/>
+    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="448">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -103,7 +103,12 @@
   <si>
     <t>"meta" : {
     "lastUpdated" : "2024-02-23T00:00:00Z",
-    "profile" : ["http://shinny.org/us/ny/hrsn/StructureDefinition/SHINNYBundleProfile"]
+    "profile" : ["http://shinny.org/us/ny/hrsn/StructureDefinition/SHINNYBundleProfile"],
+    "security": [ {
+                  "code": "ETH",
+                  "system": "http://terminology.hl7.org/CodeSystem/v3-ActCode",
+                  "display": "Substance abuse information sensitivity"
+              } ]
   },</t>
   </si>
   <si>
@@ -113,6 +118,56 @@
     <t>"http://shinny.org/us/ny/hrsn/StructureDefinition/SHINNYBundleProfile"</t>
   </si>
   <si>
+    <t>meta -&gt; security</t>
+  </si>
+  <si>
+    <r>
+      <t>If the header variable `</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X-TechBD-Part2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>` has the value '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>True</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>', then only the meta -&gt; security will be added.</t>
+    </r>
+  </si>
+  <si>
     <t>type</t>
   </si>
   <si>
@@ -128,7 +183,7 @@
     <t>entry</t>
   </si>
   <si>
-    <t>Resources - Patient, Encounter, Organization, Consent, Sexual orientation Observation , Observations, Grouper Observation</t>
+    <t>Resources - Patient, Encounter, Organization, Consent, Sexual orientation, Observations, Grouper Observation, Location</t>
   </si>
   <si>
     <t>FHIR Resources</t>
@@ -360,6 +415,13 @@
   </si>
   <si>
     <t>Observation (Observation Grouper)</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>The Location details are taken from Document.componentOf.encompassingEncounter.location.healthCareFacility.location.
+If it is not present in the CCDA file, the location details will be taken from the first occurance of the ClinicalDocument.component.structuredBody.component.section[code[@code='46240-8']].entry[1].encounter.participant.participantRole.</t>
   </si>
   <si>
     <t>Remarks</t>
@@ -1799,7 +1861,7 @@
         <scheme val="minor"/>
       </rPr>
       <t>' then, a consent resource with provision.type = "permit" will be generated. Otherwise, a consent resource with provision.type = "deny" will be generated.
-If no Observation with code **`105511-0`** is present, then `ClinicalDocument.authorization.consent[code.code='59284-0']` is evaluated:  
+If no Observation with code `105511-0` is present, then `ClinicalDocument.authorization.consent[code.code='59284-0']` is evaluated:  
   - If `displayName = "yes"`, the Consent is set to "permit".  
   - Otherwise, the Consent is set to "deny".
 If neither of the above values is available, the Consent defaults to "deny".</t>
@@ -2503,9 +2565,9 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>First preference will got to ClinicalDocument/ccda:component/ccda:structuredBody/ccda:component/ccda:section[@ID='encounters']/ccda:entry[1]/ccda:encounter[1]/ccda:statusCode/@code
+      <t>First preference will got to "ClinicalDocument/ccda:component/ccda:structuredBody/ccda:component/ccda:section[@ID='encounters']/ccda:entry[1]/ccda:encounter[1]/ccda:statusCode/@code"
 If the above path is not present, the `moodCode` is evaluated from:  
-ClinicalDocument/ccda:component/ccda:structuredBody/ccda:component/ccda:section[@ID='encounters']/ccda:entry[1]/ccda:encounter[1]/@moodCode
+"ClinicalDocument/ccda:component/ccda:structuredBody/ccda:component/ccda:section[@ID='encounters']/ccda:entry[1]/ccda:encounter[1]/@moodCode"
   - If `moodCode = '</t>
     </r>
     <r>
@@ -4163,6 +4225,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Combine the Facility ID obtained from the header variable '</t>
     </r>
     <r>
@@ -5453,9 +5522,6 @@
     <t>Included references to all the Observation resources.</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -5591,7 +5657,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5664,6 +5730,12 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -5820,6 +5892,7 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5827,23 +5900,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5873,6 +5929,22 @@
       <color rgb="FF00B050"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -6207,16 +6279,13 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -6225,119 +6294,122 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6395,9 +6467,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -6411,6 +6480,21 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -6959,20 +7043,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="25"/>
-    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
-    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="8.88181818181818" style="29"/>
+    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
+    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="25">
+      <c r="A3" s="29">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -6983,7 +7067,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="25">
+      <c r="A4" s="29">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -6994,7 +7078,7 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="25">
+      <c r="A5" s="29">
         <v>3</v>
       </c>
       <c r="B5" s="17" t="s">
@@ -7005,10 +7089,10 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="25">
+      <c r="A6" s="29">
         <v>4</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -7016,10 +7100,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="25">
+      <c r="A7" s="29">
         <v>5</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="31" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -7036,14 +7120,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7060,18 +7144,18 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="29" customHeight="1" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>424</v>
+        <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -7082,10 +7166,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="4" ht="60" spans="2:7">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="4" ht="58" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7093,7 +7177,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -7103,140 +7187,140 @@
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="29" spans="2:6">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="5" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="D7" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="120" spans="2:5">
+    <row r="8" customFormat="1" ht="116" spans="2:5">
       <c r="B8" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" ht="60" spans="2:5">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="58" spans="2:5">
       <c r="B9" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="4"/>
     </row>
     <row r="10" customFormat="1" spans="2:5">
       <c r="B10" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" customFormat="1" spans="2:5">
       <c r="B11" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="4"/>
     </row>
     <row r="12" customFormat="1" spans="2:5">
       <c r="B12" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="4"/>
     </row>
     <row r="13" customFormat="1" spans="2:5">
       <c r="B13" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="4"/>
     </row>
     <row r="14" customFormat="1" spans="2:5">
       <c r="B14" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" customFormat="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="4"/>
     </row>
     <row r="16" customFormat="1" spans="2:6">
       <c r="B16" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" customFormat="1" ht="60" customHeight="1" spans="2:6">
       <c r="B17" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
@@ -7256,15 +7340,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
-    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
+    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7292,7 +7376,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" customFormat="1" spans="1:3">
       <c r="A3" s="1"/>
       <c r="B3" t="s">
         <v>14</v>
@@ -7301,7 +7385,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" customFormat="1" spans="1:4">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
         <v>16</v>
@@ -7313,116 +7397,139 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" ht="90" spans="2:4">
-      <c r="B5" t="s">
+    <row r="5" s="24" customFormat="1" ht="61" customHeight="1" spans="1:4">
+      <c r="A5" s="25"/>
+      <c r="B5" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="26" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="2:4">
-      <c r="B6" t="s">
+    <row r="6" s="24" customFormat="1" ht="49" customHeight="1" spans="1:4">
+      <c r="A6" s="25"/>
+      <c r="B6" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="2:4">
-      <c r="B7" t="s">
+      <c r="D6" s="26"/>
+    </row>
+    <row r="7" s="24" customFormat="1" ht="86" customHeight="1" spans="1:4">
+      <c r="A7" s="25"/>
+      <c r="B7" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="2:3">
+      <c r="D7" s="26"/>
+    </row>
+    <row r="8" customFormat="1" spans="2:4">
       <c r="B8" t="s">
         <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" ht="30" spans="2:3">
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" customFormat="1" spans="2:3">
       <c r="B9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="10" customFormat="1" ht="29" spans="2:3">
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="2:3">
       <c r="B15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" ht="75" spans="2:3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" ht="72.5" spans="2:3">
       <c r="B16" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="2:3">
       <c r="B17" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" ht="75" spans="2:5">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" ht="72.5" spans="2:5">
       <c r="B18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" ht="45" spans="2:5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" ht="29" spans="2:5">
       <c r="B19" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E19" s="10"/>
     </row>
-    <row r="20" ht="45" spans="2:5">
+    <row r="20" ht="43.5" spans="2:5">
       <c r="B20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="30" spans="2:5">
+    <row r="21" ht="29" spans="2:5">
       <c r="B21" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E21" s="8"/>
     </row>
+    <row r="22" ht="101.5" spans="2:3">
+      <c r="B22" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D5:D7"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C6" r:id="rId1" display="&quot;http://shinny.org/us/ny/hrsn/StructureDefinition/SHINNYBundleProfile&quot;"/>
   </hyperlinks>
@@ -7435,13 +7542,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7449,25 +7556,25 @@
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>46</v>
+      <c r="E1" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7476,7 +7583,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="2:4">
@@ -7487,7 +7594,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -7496,7 +7603,7 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="2:3">
@@ -7504,658 +7611,658 @@
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" ht="30" spans="2:4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" ht="29" spans="2:4">
       <c r="B7" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" ht="60" spans="2:5">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" ht="58" spans="2:5">
       <c r="B8" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="2:4">
       <c r="B9" s="10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D9" s="10"/>
     </row>
     <row r="10" spans="2:4">
       <c r="B10" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="2:4">
       <c r="B11" s="15" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="2:4">
       <c r="B12" s="15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" ht="60" spans="2:4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" ht="58" spans="2:4">
       <c r="B13" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" ht="30" spans="2:4">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" ht="29" spans="2:4">
       <c r="B14" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" ht="30" spans="2:4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" ht="29" spans="2:4">
       <c r="B15" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="2:4">
       <c r="B16" s="15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" ht="120" spans="2:5">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" ht="116" spans="2:5">
       <c r="B17" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="18" ht="60" spans="2:4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" ht="58" spans="2:4">
       <c r="B18" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D18" s="12"/>
     </row>
     <row r="19" spans="2:4">
       <c r="B19" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D19" s="12"/>
     </row>
     <row r="20" spans="2:4">
       <c r="B20" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D20" s="12"/>
     </row>
     <row r="21" spans="2:4">
       <c r="B21" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D21" s="12"/>
     </row>
     <row r="22" spans="2:4">
       <c r="B22" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D22" s="12"/>
     </row>
     <row r="23" spans="2:4">
       <c r="B23" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D23" s="12"/>
     </row>
     <row r="24" ht="48" customHeight="1" spans="2:5">
       <c r="B24" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="2:3">
       <c r="B25" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" ht="198" customHeight="1" spans="2:5">
       <c r="B26" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="27" ht="45" spans="2:5">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" ht="43.5" spans="2:5">
       <c r="B27" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="28" ht="30" spans="2:5">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5">
       <c r="B28" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" ht="30" spans="2:5">
+    <row r="30" spans="2:5">
       <c r="B30" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" ht="45" spans="2:5">
+    <row r="32" ht="43.5" spans="2:5">
       <c r="B32" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="33" ht="30" spans="2:4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4">
       <c r="B33" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D33" s="14"/>
     </row>
     <row r="34" spans="2:4">
       <c r="B34" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" ht="30" spans="2:4">
+    <row r="35" spans="2:4">
       <c r="B35" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D35" s="14"/>
     </row>
     <row r="36" spans="2:4">
       <c r="B36" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D36" s="14"/>
     </row>
     <row r="37" spans="2:4">
       <c r="B37" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="38" ht="45" spans="2:5">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="38" ht="43.5" spans="2:5">
       <c r="B38" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D38" s="14"/>
-      <c r="E38" s="28" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="39" ht="120" spans="2:6">
+      <c r="E38" s="32" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="39" ht="116" spans="2:6">
       <c r="B39" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="40" ht="120" spans="2:6">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40" ht="116" spans="2:6">
       <c r="B40" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="41" spans="2:4">
       <c r="B41" s="15" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D41" s="10"/>
     </row>
     <row r="42" spans="2:4">
       <c r="B42" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D42" s="10"/>
     </row>
     <row r="43" spans="2:4">
       <c r="B43" s="15" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="2:4">
       <c r="B44" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="195" spans="2:5">
+    <row r="45" ht="188.5" spans="2:5">
       <c r="B45" s="15" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="46" ht="195" spans="2:5">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" ht="188.5" spans="2:5">
       <c r="B46" s="15" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="47" ht="195" spans="2:5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="47" ht="188.5" spans="2:5">
       <c r="B47" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="E47" s="23"/>
+        <v>153</v>
+      </c>
+      <c r="E47" s="22"/>
     </row>
     <row r="48" customFormat="1" spans="2:5">
       <c r="B48" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D48" s="10"/>
       <c r="E48" s="4"/>
     </row>
     <row r="49" customFormat="1" spans="2:5">
       <c r="B49" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D49" s="10"/>
       <c r="E49" s="4"/>
     </row>
     <row r="50" customFormat="1" spans="2:5">
       <c r="B50" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D50" s="10"/>
       <c r="E50" s="4"/>
     </row>
     <row r="51" customFormat="1" spans="2:5">
       <c r="B51" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="150" spans="2:5">
+    <row r="52" ht="145" spans="2:5">
       <c r="B52" s="10" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="2:5">
       <c r="B53" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D53" s="10"/>
       <c r="E53" s="8"/>
     </row>
     <row r="54" customFormat="1" spans="2:5">
       <c r="B54" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" customFormat="1" spans="2:5">
       <c r="B55" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D55" s="10"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" customFormat="1" spans="2:5">
       <c r="B56" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D56" s="10"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" customFormat="1" spans="2:5">
       <c r="B57" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D57" s="10"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="180" spans="2:5">
+    <row r="59" ht="174" spans="2:5">
       <c r="B59" s="10" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="60" ht="255" spans="2:6">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="60" ht="246.5" spans="2:6">
       <c r="B60" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="61" spans="2:6">
       <c r="B61" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D61" s="10"/>
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="2:6">
       <c r="B62" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="210" spans="2:6">
+    <row r="63" ht="203" spans="2:6">
       <c r="B63" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D63" s="10"/>
       <c r="E63" s="13" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F63" s="4"/>
     </row>
     <row r="64" ht="56" customHeight="1" spans="2:6">
       <c r="B64" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="65" ht="43" customHeight="1" spans="2:4">
       <c r="B65" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D65" s="12"/>
     </row>
     <row r="66" ht="40" customHeight="1" spans="2:4">
       <c r="B66" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D66" s="12"/>
     </row>
     <row r="67" spans="2:4">
       <c r="B67" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="68" ht="43" customHeight="1" spans="2:4">
       <c r="B68" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D68" s="14"/>
     </row>
@@ -8178,14 +8285,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8202,18 +8309,18 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="105" customHeight="1" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -8224,10 +8331,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="4" ht="60" spans="2:7">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" ht="58" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8235,7 +8342,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -8245,7 +8352,7 @@
         <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E5" s="8"/>
     </row>
@@ -8254,210 +8361,210 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>197</v>
-      </c>
-      <c r="E6" s="24"/>
-    </row>
-    <row r="7" ht="120" spans="2:6">
+        <v>201</v>
+      </c>
+      <c r="E6" s="23"/>
+    </row>
+    <row r="7" ht="116" spans="2:6">
       <c r="B7" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F7" s="4"/>
     </row>
     <row r="8" ht="94" customHeight="1" spans="2:5">
       <c r="B8" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C8" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" customFormat="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C9" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="5" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C10" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="11" ht="225" spans="2:5">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" ht="203" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C12" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="5" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="14" ht="45" spans="2:5">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" ht="43.5" spans="2:5">
       <c r="B14" s="5" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D14" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="15" ht="255" spans="2:5">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" ht="246.5" spans="2:5">
       <c r="B15" s="5" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="16" ht="45" spans="2:5">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" ht="43.5" spans="2:5">
       <c r="B16" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C16" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="45" spans="2:5">
+    <row r="17" ht="43.5" spans="2:5">
       <c r="B17" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C17" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="45" spans="2:5">
+    <row r="18" ht="43.5" spans="2:5">
       <c r="B18" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C18" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="19" ht="60" spans="2:5">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" ht="58" spans="2:5">
       <c r="B19" s="5" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C19" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="2:5">
       <c r="B20" s="5" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C20" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="8" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" customFormat="1" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E21" s="8"/>
       <c r="F21" s="4"/>
     </row>
     <row r="22" customFormat="1" ht="60" customHeight="1" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="8"/>
@@ -8478,14 +8585,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="42.2857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
+    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8495,7 +8602,7 @@
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -8510,10 +8617,10 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -8524,10 +8631,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="4" ht="75" spans="1:5">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="4" ht="72.5" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8536,10 +8643,10 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -8548,226 +8655,226 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="255" spans="2:5">
+    <row r="7" ht="246.5" spans="2:5">
       <c r="B7" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D7" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" ht="71" customHeight="1" spans="2:5">
       <c r="B8" s="5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="30" spans="2:5">
+    <row r="9" ht="29" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D9" s="10"/>
-      <c r="E9" s="23"/>
+      <c r="E9" s="22"/>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="5" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="30" spans="2:4">
+    <row r="11" ht="29" spans="2:4">
       <c r="B11" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="12" ht="60" spans="2:5">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="12" ht="58" spans="2:5">
       <c r="B12" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="13" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" ht="33" customHeight="1" spans="2:4">
       <c r="B13" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" customFormat="1" spans="2:3">
       <c r="B14" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" ht="60" spans="2:4">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" ht="58" spans="2:4">
       <c r="B15" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C15" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="16" customFormat="1" ht="30" spans="2:3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="16" customFormat="1" ht="29" spans="2:3">
       <c r="B16" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="17" ht="60" spans="2:4">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="17" ht="58" spans="2:4">
       <c r="B17" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" spans="2:3">
       <c r="B18" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="19" ht="45" spans="2:5">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="19" ht="43.5" spans="2:5">
       <c r="B19" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="E20" s="17"/>
     </row>
     <row r="21" ht="409.5" spans="2:5">
       <c r="B21" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="22" ht="60" spans="2:5">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="22" ht="58" spans="2:5">
       <c r="B22" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="E22" s="21"/>
+        <v>288</v>
+      </c>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" ht="66" customHeight="1" spans="2:5">
       <c r="B23" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C23" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24" customFormat="1" spans="2:5">
       <c r="B24" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D24" s="10"/>
       <c r="E24" s="4"/>
     </row>
     <row r="25" customFormat="1" spans="2:4">
       <c r="B25" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
     </row>
     <row r="26" customFormat="1" ht="46" customHeight="1" spans="2:4">
       <c r="B26" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D26" s="14"/>
     </row>
@@ -8789,14 +8896,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
-    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
+    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8813,15 +8920,15 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="1" spans="2:3">
@@ -8829,7 +8936,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" spans="2:3">
@@ -8846,20 +8953,20 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -8867,270 +8974,270 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="5" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D7" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
     </row>
     <row r="8" ht="63" customHeight="1" spans="2:6">
       <c r="B8" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>301</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>302</v>
+        <v>305</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="30" spans="2:5">
+    <row r="10" ht="29" spans="2:5">
       <c r="B10" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="30" spans="2:5">
+    <row r="11" ht="29" spans="2:5">
       <c r="B11" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:5">
+    <row r="12" ht="29" spans="2:5">
       <c r="B12" s="4" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="8"/>
     </row>
     <row r="13" customFormat="1" ht="66" customHeight="1" spans="2:6">
       <c r="B13" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>312</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>302</v>
+        <v>316</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="14" customFormat="1" spans="2:5">
       <c r="B14" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="D14" s="10"/>
-      <c r="E14" s="21"/>
-    </row>
-    <row r="15" customFormat="1" ht="30" spans="2:5">
+      <c r="E14" s="20"/>
+    </row>
+    <row r="15" customFormat="1" ht="29" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="D15" s="10"/>
-      <c r="E15" s="21"/>
-    </row>
-    <row r="16" customFormat="1" ht="30" spans="2:5">
+      <c r="E15" s="20"/>
+    </row>
+    <row r="16" customFormat="1" ht="29" spans="2:5">
       <c r="B16" s="4" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="30" spans="2:4">
+    <row r="17" customFormat="1" ht="29" spans="2:4">
       <c r="B17" s="4" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="60" spans="2:5">
+    <row r="18" ht="58" spans="2:5">
       <c r="B18" s="5" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="19" ht="93" customHeight="1" spans="2:6">
       <c r="B19" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="2:6">
       <c r="B20" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="10"/>
       <c r="F20" s="8" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="21" customFormat="1" ht="50" customHeight="1" spans="2:6">
       <c r="B21" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="10" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="30" spans="2:6">
+    <row r="22" customFormat="1" ht="29" spans="2:6">
       <c r="B22" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="195" spans="2:6">
+    <row r="23" customFormat="1" ht="188.5" spans="2:6">
       <c r="B23" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="13" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="120" spans="2:6">
+    <row r="24" customFormat="1" ht="116" spans="2:6">
       <c r="B24" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="30" spans="2:6">
+    <row r="25" customFormat="1" ht="29" spans="2:6">
       <c r="B25" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D25" s="10"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="30" spans="2:6">
+    <row r="26" customFormat="1" ht="29" spans="2:6">
       <c r="B26" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="30" spans="2:6">
+    <row r="27" customFormat="1" ht="29" spans="2:6">
       <c r="B27" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D27" s="10"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="30" spans="2:6">
+    <row r="28" customFormat="1" ht="29" spans="2:6">
       <c r="B28" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="30" spans="2:6">
+    <row r="29" customFormat="1" ht="29" spans="2:6">
       <c r="B29" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="30" spans="2:6">
+    <row r="30" customFormat="1" ht="29" spans="2:6">
       <c r="B30" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D30" s="10"/>
       <c r="E30" s="4"/>
@@ -9138,21 +9245,21 @@
     </row>
     <row r="31" customFormat="1" spans="2:4">
       <c r="B31" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="32" customFormat="1" ht="46" customHeight="1" spans="2:4">
       <c r="B32" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D32" s="14"/>
     </row>
@@ -9174,13 +9281,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="46.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
-    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
+    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
+    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9198,15 +9305,15 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" ht="45" spans="1:1">
-      <c r="A2" s="20" t="s">
-        <v>342</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" ht="43.5" spans="1:1">
+      <c r="A2" s="19" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -9215,7 +9322,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9227,7 +9334,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -9236,18 +9343,18 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9255,161 +9362,161 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="8" ht="150" spans="2:5">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" ht="145" spans="2:5">
       <c r="B8" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="D8" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1" spans="2:4">
       <c r="B9" s="5" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="10" ht="30" spans="2:4">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="10" ht="29" spans="2:4">
       <c r="B10" s="5" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D10" s="10"/>
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:4">
+    <row r="12" ht="29" spans="2:4">
       <c r="B12" s="5" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D12" s="10"/>
     </row>
     <row r="13" ht="38" customHeight="1" spans="2:4">
       <c r="B13" s="4" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="14" ht="30" spans="2:4">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="14" ht="29" spans="2:4">
       <c r="B14" s="4" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D14" s="10"/>
     </row>
     <row r="15" ht="153" customHeight="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="8" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="16" ht="75" spans="2:4">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="16" ht="58" spans="2:4">
       <c r="B16" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C16" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="17" ht="30" spans="2:3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17" ht="29" spans="2:3">
       <c r="B17" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="18" ht="90" spans="2:5">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="18" ht="87" spans="2:5">
       <c r="B18" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="D18" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
     </row>
     <row r="19" spans="2:6">
       <c r="B19" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D19" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="20" spans="2:4">
       <c r="B20" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1" spans="2:4">
       <c r="B21" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D21" s="14"/>
     </row>
@@ -9428,14 +9535,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9452,18 +9559,18 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="17" customHeight="1" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9476,19 +9583,19 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="4" ht="78" spans="1:5">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="4" ht="82.5" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>376</v>
+        <v>379</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>380</v>
       </c>
       <c r="E4" s="16"/>
     </row>
@@ -9498,18 +9605,18 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9517,270 +9624,270 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="8" ht="150" spans="2:5">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" ht="145" spans="2:5">
       <c r="B8" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="D8" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" ht="139" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="10" ht="45" spans="2:5">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="10" ht="43.5" spans="2:5">
       <c r="B10" s="5" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="11" ht="210" spans="2:5">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="11" ht="203" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="11" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="12" ht="210" spans="2:5">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="12" ht="203" spans="2:5">
       <c r="B12" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="11" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="5" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1" spans="2:5">
       <c r="B14" s="5" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="5" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="9"/>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="30" spans="2:5">
+    <row r="17" ht="29" spans="2:5">
       <c r="B17" s="5" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="8" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="18" ht="105" spans="2:5">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="18" ht="101.5" spans="2:5">
       <c r="B18" s="4" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="19" ht="30" spans="2:3">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="19" ht="29" spans="2:3">
       <c r="B19" s="4" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="20" ht="30" spans="2:3">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="20" ht="29" spans="2:3">
       <c r="B20" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C20" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" ht="37" customHeight="1" spans="2:5">
       <c r="B21" s="5" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="75" spans="2:5">
+    <row r="22" ht="72.5" spans="2:5">
       <c r="B22" s="5" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C22" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="11" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="23" ht="45" spans="2:5">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="23" ht="43.5" spans="2:5">
       <c r="B23" s="5" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="11" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="24" ht="75" spans="2:4">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="24" ht="58" spans="2:4">
       <c r="B24" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C24" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="25" ht="30" spans="2:3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="25" ht="29" spans="2:3">
       <c r="B25" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="26" ht="45" spans="2:4">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="26" ht="43.5" spans="2:4">
       <c r="B26" s="5" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="C26" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="27" ht="210" spans="2:5">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="27" ht="203" spans="2:5">
       <c r="B27" s="5" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="28" ht="45" spans="2:4">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="28" ht="43.5" spans="2:4">
       <c r="B28" s="5" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D29" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="30" spans="2:4">
       <c r="B30" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
     <row r="31" ht="46" customHeight="1" spans="2:4">
       <c r="B31" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D31" s="14"/>
     </row>
@@ -9801,14 +9908,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9825,18 +9932,18 @@
         <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9849,7 +9956,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9861,7 +9968,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -9870,18 +9977,18 @@
         <v>19</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9889,170 +9996,170 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="8" ht="150" spans="2:5">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" ht="145" spans="2:5">
       <c r="B8" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="D8" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" ht="409" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="10" ht="165" spans="2:5">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="10" ht="159.5" spans="2:5">
       <c r="B10" s="5" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="11" ht="180" spans="2:5">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="11" ht="159.5" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C11" s="4"/>
       <c r="E11" s="11" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="12" ht="150" spans="2:5">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="12" ht="145" spans="2:5">
       <c r="B12" s="5" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C12" s="4"/>
       <c r="E12" s="11" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="13" ht="75" spans="2:4">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="13" ht="58" spans="2:4">
       <c r="B13" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C13" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="14" ht="30" spans="2:3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" ht="29" spans="2:3">
       <c r="B14" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="15" ht="45" spans="2:4">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="15" ht="43.5" spans="2:4">
       <c r="B15" s="5" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="C15" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="16" ht="210" spans="2:5">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="16" ht="203" spans="2:5">
       <c r="B16" s="5" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="17" ht="45" spans="2:4">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="17" ht="43.5" spans="2:4">
       <c r="B17" s="5" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="18" spans="2:6">
       <c r="B18" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D18" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="19" ht="165" spans="2:5">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="19" ht="159.5" spans="2:5">
       <c r="B19" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="E19" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
     </row>
     <row r="20" spans="2:4">
       <c r="B20" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1" spans="2:4">
       <c r="B21" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D21" s="14"/>
     </row>

</xml_diff>

<commit_message>
feat: update XSLT files to add more values for ddress.use and telecom.use in Patient, Organization, and Location Resources of CCDA and HL7 files #2841 - Updated XSLT files to add more values for ddress.use and telecom.use in Patient, Organization, and Location Resources of CCDA and HL7 files - Updated the FHIR conversion specification documents for CCDA and HL7 with the changes in address and telecom use
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="449">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -122,6 +122,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>If the header variable `</t>
     </r>
     <r>
@@ -625,13 +632,11 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-HP -&gt; home  
-H -&gt; home  
-WP -&gt; work  
-TMP -&gt; temp  
-OLD -&gt; old  
-BAD -&gt; old  
-All Others -&gt; patientRole.addr.use</t>
+WP, DIR, PUB -&gt; work
+BA -&gt; billing
+TMP -&gt; temp
+OLD, BAD -&gt; old
+All Others -&gt; home</t>
     </r>
   </si>
   <si>
@@ -722,18 +727,12 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-AS -&gt; work  
-DIR -&gt; work  
-PUB -&gt; work  
-WP -&gt; work  
-BAD -&gt; old  
-H -&gt; home  
-HP -&gt; home  
-HV -&gt; home  
-MC -&gt; mobile  
-PG -&gt; mobile  
-TMP -&gt; temp  
-All Others -&gt; patient.telecom.use</t>
+AS, DIR, PUB, WP, WPN -&gt; work
+H, HP, HV, PRN, ORN, PRS -&gt; home
+MC, PG -&gt; mobile
+TMP -&gt; temp
+BAD -&gt; old
+All others -&gt; home</t>
     </r>
   </si>
   <si>
@@ -3828,6 +3827,35 @@
     <t>Document.author.assignedAuthor.representedOrganization.telecom.use</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>telecom -&gt; use Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+AS, DIR, PUB, WP, WPN -&gt; work
+MC, PG -&gt; mobile
+TMP -&gt; temp
+BAD -&gt; old
+All others -&gt; work</t>
+    </r>
+  </si>
+  <si>
     <t>Document.author.assignedAuthor.representedOrganization.addr.streetAddressLine
 Document.author.assignedAuthor.representedOrganization.addr.city
 Document.author.assignedAuthor.representedOrganization.addr.state,
@@ -3846,6 +3874,35 @@
   </si>
   <si>
     <t>Document.author.assignedAuthor.representedOrganization.addr.use</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>addr.use -&gt; use Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+WP, DIR, PUB -&gt; work
+BA -&gt; billing
+TMP -&gt; temp
+OLD, BAD -&gt; old
+All Others -&gt; work</t>
+    </r>
   </si>
   <si>
     <t>Document.author.assignedAuthor.representedOrganization.addr.streetAddressLine</t>
@@ -5578,37 +5635,6 @@
   </si>
   <si>
     <t>addr.use</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>addr.use -&gt; use Mapping</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-HP -&gt; home  
-H -&gt; home  
-WP -&gt; work  
-TMP -&gt; temp  
-OLD -&gt; old  
-BAD -&gt; old  
-All Others -&gt;addr.use</t>
-    </r>
   </si>
   <si>
     <t>addr.streetAddressLine
@@ -5892,7 +5918,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5900,6 +5925,7 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6409,7 +6435,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6471,6 +6497,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7043,20 +7072,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88181818181818" style="29"/>
-    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
-    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
+    <col min="1" max="1" width="8.88571428571429" style="30"/>
+    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
+    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="31" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="29">
+      <c r="A3" s="30">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -7067,7 +7096,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="29">
+      <c r="A4" s="30">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -7078,7 +7107,7 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="29">
+      <c r="A5" s="30">
         <v>3</v>
       </c>
       <c r="B5" s="17" t="s">
@@ -7089,10 +7118,10 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="29">
+      <c r="A6" s="30">
         <v>4</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="24" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -7100,10 +7129,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="29">
+      <c r="A7" s="30">
         <v>5</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="32" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -7120,14 +7149,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7155,7 +7184,7 @@
         <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -7166,10 +7195,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="4" ht="58" spans="2:7">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="4" ht="60" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7177,7 +7206,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -7191,18 +7220,18 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="29" spans="2:6">
+    <row r="6" ht="30" spans="2:6">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="7" spans="2:6">
@@ -7210,34 +7239,34 @@
         <v>324</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D7" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="116" spans="2:5">
+    <row r="8" customFormat="1" ht="90" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>86</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" ht="58" spans="2:5">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="60" spans="2:5">
       <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="4"/>
@@ -7247,7 +7276,7 @@
         <v>90</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="4"/>
@@ -7257,7 +7286,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="4"/>
@@ -7267,7 +7296,7 @@
         <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="4"/>
@@ -7277,7 +7306,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="4"/>
@@ -7287,17 +7316,17 @@
         <v>98</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" customFormat="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="4"/>
@@ -7310,7 +7339,7 @@
         <v>193</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
@@ -7320,7 +7349,7 @@
         <v>195</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
@@ -7341,14 +7370,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
-    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
+    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7397,37 +7426,37 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" s="24" customFormat="1" ht="61" customHeight="1" spans="1:4">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25" t="s">
+    <row r="5" s="25" customFormat="1" ht="61" customHeight="1" spans="1:4">
+      <c r="A5" s="26"/>
+      <c r="B5" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" s="24" customFormat="1" ht="49" customHeight="1" spans="1:4">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25" t="s">
+    <row r="6" s="25" customFormat="1" ht="49" customHeight="1" spans="1:4">
+      <c r="A6" s="26"/>
+      <c r="B6" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="26"/>
-    </row>
-    <row r="7" s="24" customFormat="1" ht="86" customHeight="1" spans="1:4">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25" t="s">
+      <c r="D6" s="27"/>
+    </row>
+    <row r="7" s="25" customFormat="1" ht="86" customHeight="1" spans="1:4">
+      <c r="A7" s="26"/>
+      <c r="B7" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="26"/>
+      <c r="D7" s="27"/>
     </row>
     <row r="8" customFormat="1" spans="2:4">
       <c r="B8" t="s">
@@ -7446,7 +7475,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="29" spans="2:3">
+    <row r="10" customFormat="1" ht="30" spans="2:3">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7467,7 +7496,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="72.5" spans="2:3">
+    <row r="16" ht="75" spans="2:3">
       <c r="B16" t="s">
         <v>35</v>
       </c>
@@ -7483,7 +7512,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="72.5" spans="2:5">
+    <row r="18" ht="75" spans="2:5">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -7494,7 +7523,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="29" spans="2:5">
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
@@ -7503,7 +7532,7 @@
       </c>
       <c r="E19" s="10"/>
     </row>
-    <row r="20" ht="43.5" spans="2:5">
+    <row r="20" ht="45" spans="2:5">
       <c r="B20" t="s">
         <v>44</v>
       </c>
@@ -7512,14 +7541,14 @@
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="29" spans="2:5">
+    <row r="21" ht="30" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="101.5" spans="2:3">
-      <c r="B22" s="28" t="s">
+    <row r="22" ht="105" spans="2:3">
+      <c r="B22" s="29" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="10" t="s">
@@ -7542,13 +7571,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7556,19 +7585,19 @@
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="22" t="s">
         <v>50</v>
       </c>
     </row>
@@ -7614,7 +7643,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="29" spans="2:4">
+    <row r="7" ht="30" spans="2:4">
       <c r="B7" s="4" t="s">
         <v>55</v>
       </c>
@@ -7625,7 +7654,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" ht="58" spans="2:5">
+    <row r="8" ht="60" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
@@ -7681,7 +7710,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" ht="58" spans="2:4">
+    <row r="13" ht="60" spans="2:4">
       <c r="B13" s="4" t="s">
         <v>72</v>
       </c>
@@ -7692,7 +7721,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" ht="29" spans="2:4">
+    <row r="14" ht="30" spans="2:4">
       <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
@@ -7703,7 +7732,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" ht="29" spans="2:4">
+    <row r="15" ht="30" spans="2:4">
       <c r="B15" s="4" t="s">
         <v>78</v>
       </c>
@@ -7725,7 +7754,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" ht="116" spans="2:5">
+    <row r="17" ht="90" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>84</v>
       </c>
@@ -7739,7 +7768,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="58" spans="2:4">
+    <row r="18" ht="60" spans="2:4">
       <c r="B18" s="4" t="s">
         <v>88</v>
       </c>
@@ -7812,18 +7841,18 @@
         <v>104</v>
       </c>
     </row>
-    <row r="26" ht="198" customHeight="1" spans="2:5">
+    <row r="26" ht="105" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>105</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="21" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="27" ht="43.5" spans="2:5">
+    <row r="27" ht="45" spans="2:5">
       <c r="B27" s="4" t="s">
         <v>108</v>
       </c>
@@ -7837,7 +7866,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="2:5">
+    <row r="28" ht="30" spans="2:5">
       <c r="B28" s="4" t="s">
         <v>112</v>
       </c>
@@ -7857,7 +7886,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="2:5">
+    <row r="30" ht="30" spans="2:5">
       <c r="B30" s="4" t="s">
         <v>116</v>
       </c>
@@ -7877,7 +7906,7 @@
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" ht="43.5" spans="2:5">
+    <row r="32" ht="45" spans="2:5">
       <c r="B32" s="4" t="s">
         <v>108</v>
       </c>
@@ -7891,7 +7920,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="2:4">
+    <row r="33" ht="30" spans="2:4">
       <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
@@ -7909,7 +7938,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" spans="2:4">
+    <row r="35" ht="30" spans="2:4">
       <c r="B35" s="4" t="s">
         <v>116</v>
       </c>
@@ -7938,7 +7967,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" ht="43.5" spans="2:5">
+    <row r="38" ht="45" spans="2:5">
       <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
@@ -7946,11 +7975,11 @@
         <v>79</v>
       </c>
       <c r="D38" s="14"/>
-      <c r="E38" s="32" t="s">
+      <c r="E38" s="33" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="39" ht="116" spans="2:6">
+    <row r="39" ht="120" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>130</v>
       </c>
@@ -7961,7 +7990,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" ht="116" spans="2:6">
+    <row r="40" ht="120" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>133</v>
       </c>
@@ -8008,7 +8037,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="188.5" spans="2:5">
+    <row r="45" ht="195" spans="2:5">
       <c r="B45" s="15" t="s">
         <v>143</v>
       </c>
@@ -8022,7 +8051,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" ht="188.5" spans="2:5">
+    <row r="46" ht="195" spans="2:5">
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
@@ -8036,7 +8065,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" ht="188.5" spans="2:5">
+    <row r="47" ht="195" spans="2:5">
       <c r="B47" s="15" t="s">
         <v>151</v>
       </c>
@@ -8046,7 +8075,7 @@
       <c r="D47" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E47" s="22"/>
+      <c r="E47" s="23"/>
     </row>
     <row r="48" customFormat="1" spans="2:5">
       <c r="B48" s="4" t="s">
@@ -8088,7 +8117,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="145" spans="2:5">
+    <row r="52" ht="150" spans="2:5">
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
@@ -8162,7 +8191,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="174" spans="2:5">
+    <row r="59" ht="180" spans="2:5">
       <c r="B59" s="10" t="s">
         <v>174</v>
       </c>
@@ -8176,7 +8205,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="60" ht="246.5" spans="2:6">
+    <row r="60" ht="255" spans="2:6">
       <c r="B60" s="4" t="s">
         <v>177</v>
       </c>
@@ -8207,7 +8236,7 @@
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="203" spans="2:6">
+    <row r="63" ht="210" spans="2:6">
       <c r="B63" s="4" t="s">
         <v>184</v>
       </c>
@@ -8285,14 +8314,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8334,7 +8363,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" ht="58" spans="2:7">
+    <row r="4" ht="60" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8363,9 +8392,9 @@
       <c r="C6" t="s">
         <v>201</v>
       </c>
-      <c r="E6" s="23"/>
-    </row>
-    <row r="7" ht="116" spans="2:6">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" ht="120" spans="2:6">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8418,7 +8447,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" ht="203" spans="2:5">
+    <row r="11" ht="225" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -8454,7 +8483,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" ht="43.5" spans="2:5">
+    <row r="14" ht="45" spans="2:5">
       <c r="B14" s="5" t="s">
         <v>221</v>
       </c>
@@ -8468,7 +8497,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" ht="246.5" spans="2:5">
+    <row r="15" ht="255" spans="2:5">
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
@@ -8482,7 +8511,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" ht="43.5" spans="2:5">
+    <row r="16" ht="45" spans="2:5">
       <c r="B16" s="5" t="s">
         <v>229</v>
       </c>
@@ -8494,7 +8523,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="43.5" spans="2:5">
+    <row r="17" ht="45" spans="2:5">
       <c r="B17" s="5" t="s">
         <v>232</v>
       </c>
@@ -8506,7 +8535,7 @@
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="43.5" spans="2:5">
+    <row r="18" ht="45" spans="2:5">
       <c r="B18" t="s">
         <v>235</v>
       </c>
@@ -8520,7 +8549,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="58" spans="2:5">
+    <row r="19" ht="60" spans="2:5">
       <c r="B19" s="5" t="s">
         <v>238</v>
       </c>
@@ -8585,14 +8614,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
-    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="42.2857142857143" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8602,7 +8631,7 @@
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -8634,7 +8663,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" ht="72.5" spans="1:5">
+    <row r="4" ht="75" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8661,7 +8690,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -8672,7 +8701,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="246.5" spans="2:5">
+    <row r="7" ht="255" spans="2:5">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8698,7 +8727,7 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="29" spans="2:5">
+    <row r="9" ht="30" spans="2:5">
       <c r="B9" s="5" t="s">
         <v>256</v>
       </c>
@@ -8706,7 +8735,7 @@
         <v>257</v>
       </c>
       <c r="D9" s="10"/>
-      <c r="E9" s="22"/>
+      <c r="E9" s="23"/>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="5" t="s">
@@ -8718,7 +8747,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="29" spans="2:4">
+    <row r="11" ht="30" spans="2:4">
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
@@ -8729,7 +8758,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" ht="58" spans="2:5">
+    <row r="12" ht="60" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>263</v>
       </c>
@@ -8755,7 +8784,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="58" spans="2:4">
+    <row r="15" customFormat="1" ht="60" spans="2:4">
       <c r="B15" s="5" t="s">
         <v>269</v>
       </c>
@@ -8766,7 +8795,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="29" spans="2:3">
+    <row r="16" customFormat="1" ht="30" spans="2:3">
       <c r="B16" s="5" t="s">
         <v>271</v>
       </c>
@@ -8774,7 +8803,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" ht="58" spans="2:4">
+    <row r="17" ht="60" spans="2:4">
       <c r="B17" t="s">
         <v>273</v>
       </c>
@@ -8793,7 +8822,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" ht="43.5" spans="2:5">
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" t="s">
         <v>278</v>
       </c>
@@ -8827,7 +8856,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="22" ht="58" spans="2:5">
+    <row r="22" ht="60" spans="2:5">
       <c r="B22" t="s">
         <v>287</v>
       </c>
@@ -8896,14 +8925,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
-    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
+    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8961,7 +8990,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -9010,7 +9039,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="29" spans="2:5">
+    <row r="10" ht="30" spans="2:5">
       <c r="B10" s="4" t="s">
         <v>309</v>
       </c>
@@ -9020,7 +9049,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="29" spans="2:5">
+    <row r="11" ht="30" spans="2:5">
       <c r="B11" s="4" t="s">
         <v>311</v>
       </c>
@@ -9030,7 +9059,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="29" spans="2:5">
+    <row r="12" ht="30" spans="2:5">
       <c r="B12" s="4" t="s">
         <v>312</v>
       </c>
@@ -9064,7 +9093,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="20"/>
     </row>
-    <row r="15" customFormat="1" ht="29" spans="2:5">
+    <row r="15" customFormat="1" ht="30" spans="2:5">
       <c r="B15" s="4" t="s">
         <v>319</v>
       </c>
@@ -9074,7 +9103,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="20"/>
     </row>
-    <row r="16" customFormat="1" ht="29" spans="2:5">
+    <row r="16" customFormat="1" ht="30" spans="2:5">
       <c r="B16" s="4" t="s">
         <v>321</v>
       </c>
@@ -9084,7 +9113,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="29" spans="2:4">
+    <row r="17" customFormat="1" ht="30" spans="2:4">
       <c r="B17" s="4" t="s">
         <v>322</v>
       </c>
@@ -9093,7 +9122,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="58" spans="2:5">
+    <row r="18" ht="60" spans="2:5">
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
@@ -9141,7 +9170,7 @@
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="29" spans="2:6">
+    <row r="22" customFormat="1" ht="30" spans="2:6">
       <c r="B22" s="4" t="s">
         <v>103</v>
       </c>
@@ -9151,7 +9180,7 @@
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="188.5" spans="2:6">
+    <row r="23" customFormat="1" ht="90" spans="2:6">
       <c r="B23" s="4" t="s">
         <v>105</v>
       </c>
@@ -9159,85 +9188,87 @@
         <v>335</v>
       </c>
       <c r="D23" s="10"/>
-      <c r="E23" s="13" t="s">
-        <v>107</v>
+      <c r="E23" s="21" t="s">
+        <v>336</v>
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="116" spans="2:6">
+    <row r="24" customFormat="1" ht="120" spans="2:6">
       <c r="B24" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="29" spans="2:6">
+    <row r="25" customFormat="1" ht="90" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D25" s="10"/>
-      <c r="E25" s="4"/>
+      <c r="E25" s="13" t="s">
+        <v>340</v>
+      </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="29" spans="2:6">
+    <row r="26" customFormat="1" ht="30" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>90</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="29" spans="2:6">
+    <row r="27" customFormat="1" ht="30" spans="2:6">
       <c r="B27" s="4" t="s">
         <v>92</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D27" s="10"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="29" spans="2:6">
+    <row r="28" customFormat="1" ht="30" spans="2:6">
       <c r="B28" s="4" t="s">
         <v>94</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="29" spans="2:6">
+    <row r="29" customFormat="1" ht="30" spans="2:6">
       <c r="B29" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="29" spans="2:6">
+    <row r="30" customFormat="1" ht="30" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D30" s="10"/>
       <c r="E30" s="4"/>
@@ -9251,7 +9282,7 @@
         <v>193</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="32" customFormat="1" ht="46" customHeight="1" spans="2:4">
@@ -9259,7 +9290,7 @@
         <v>195</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D32" s="14"/>
     </row>
@@ -9281,13 +9312,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
-    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
-    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
-    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
+    <col min="3" max="3" width="46.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
+    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9311,9 +9342,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="43.5" spans="1:1">
+    <row r="2" ht="45" spans="1:1">
       <c r="A2" s="19" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -9322,7 +9353,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9334,7 +9365,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -9349,12 +9380,12 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="29" spans="2:6">
+    <row r="6" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9368,46 +9399,46 @@
         <v>57</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" ht="145" spans="2:5">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" ht="150" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1" spans="2:4">
       <c r="B9" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="10" ht="29" spans="2:4">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="10" ht="30" spans="2:4">
       <c r="B10" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D10" s="10"/>
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>220</v>
@@ -9415,48 +9446,48 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="29" spans="2:4">
+    <row r="12" ht="30" spans="2:4">
       <c r="B12" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>360</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>358</v>
       </c>
       <c r="D12" s="10"/>
     </row>
     <row r="13" ht="38" customHeight="1" spans="2:4">
       <c r="B13" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="14" ht="29" spans="2:4">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="2:4">
       <c r="B14" s="4" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D14" s="10"/>
     </row>
     <row r="15" ht="153" customHeight="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="8" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="16" ht="58" spans="2:4">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="16" ht="75" spans="2:4">
       <c r="B16" s="5" t="s">
         <v>269</v>
       </c>
@@ -9467,7 +9498,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" ht="29" spans="2:3">
+    <row r="17" ht="30" spans="2:3">
       <c r="B17" s="5" t="s">
         <v>271</v>
       </c>
@@ -9475,29 +9506,29 @@
         <v>272</v>
       </c>
     </row>
-    <row r="18" ht="87" spans="2:5">
+    <row r="18" ht="90" spans="2:5">
       <c r="B18" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D18" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="19" spans="2:6">
       <c r="B19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D19" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="20" spans="2:4">
@@ -9508,7 +9539,7 @@
         <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1" spans="2:4">
@@ -9516,7 +9547,7 @@
         <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D21" s="14"/>
     </row>
@@ -9535,14 +9566,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9570,7 +9601,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9583,19 +9614,19 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="4" ht="82.5" spans="1:5">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="4" ht="78" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E4" s="16"/>
     </row>
@@ -9611,12 +9642,12 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -9630,90 +9661,90 @@
         <v>57</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" ht="145" spans="2:5">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" ht="150" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" ht="139" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="10" ht="43.5" spans="2:5">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="10" ht="45" spans="2:5">
       <c r="B10" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="11" ht="203" spans="2:5">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11" ht="210" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="11" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="12" ht="203" spans="2:5">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="12" ht="210" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="11" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="5" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1" spans="2:5">
       <c r="B14" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>259</v>
@@ -9723,7 +9754,7 @@
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>220</v>
@@ -9731,43 +9762,43 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="29" spans="2:5">
+    <row r="17" ht="30" spans="2:5">
       <c r="B17" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="8" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="18" ht="101.5" spans="2:5">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="18" ht="105" spans="2:5">
       <c r="B18" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="19" ht="29" spans="2:3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" ht="30" spans="2:3">
       <c r="B19" s="4" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="20" ht="29" spans="2:3">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="20" ht="30" spans="2:3">
       <c r="B20" s="4" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C20" t="s">
         <v>220</v>
@@ -9775,38 +9806,38 @@
     </row>
     <row r="21" ht="37" customHeight="1" spans="2:5">
       <c r="B21" s="5" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="72.5" spans="2:5">
+    <row r="22" ht="75" spans="2:5">
       <c r="B22" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C22" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="11" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="23" ht="43.5" spans="2:5">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="23" ht="45" spans="2:5">
       <c r="B23" s="5" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="11" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="24" ht="58" spans="2:4">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="24" ht="75" spans="2:4">
       <c r="B24" s="5" t="s">
         <v>269</v>
       </c>
@@ -9817,7 +9848,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" ht="29" spans="2:3">
+    <row r="25" ht="30" spans="2:3">
       <c r="B25" s="5" t="s">
         <v>271</v>
       </c>
@@ -9825,50 +9856,50 @@
         <v>272</v>
       </c>
     </row>
-    <row r="26" ht="43.5" spans="2:4">
+    <row r="26" ht="45" spans="2:4">
       <c r="B26" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C26" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="2:5">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="27" ht="210" spans="2:5">
       <c r="B27" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="28" ht="43.5" spans="2:4">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="28" ht="45" spans="2:4">
       <c r="B28" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D29" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="30" spans="2:4">
@@ -9879,7 +9910,7 @@
         <v>193</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="31" ht="46" customHeight="1" spans="2:4">
@@ -9887,7 +9918,7 @@
         <v>195</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D31" s="14"/>
     </row>
@@ -9908,14 +9939,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9943,7 +9974,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9956,7 +9987,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9968,7 +9999,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -9983,12 +10014,12 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -10002,70 +10033,70 @@
         <v>57</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="8" ht="145" spans="2:5">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" ht="150" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" ht="409" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="10" ht="159.5" spans="2:5">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="10" ht="165" spans="2:5">
       <c r="B10" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>254</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="11" ht="159.5" spans="2:5">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="11" ht="180" spans="2:5">
       <c r="B11" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C11" s="4"/>
       <c r="E11" s="11" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="12" ht="145" spans="2:5">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="12" ht="150" spans="2:5">
       <c r="B12" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C12" s="4"/>
       <c r="E12" s="11" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="13" ht="58" spans="2:4">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" ht="75" spans="2:4">
       <c r="B13" s="5" t="s">
         <v>269</v>
       </c>
@@ -10076,7 +10107,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" ht="29" spans="2:3">
+    <row r="14" ht="30" spans="2:3">
       <c r="B14" s="5" t="s">
         <v>271</v>
       </c>
@@ -10084,63 +10115,63 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" ht="43.5" spans="2:4">
+    <row r="15" ht="45" spans="2:4">
       <c r="B15" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C15" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="16" ht="203" spans="2:5">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="16" ht="210" spans="2:5">
       <c r="B16" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="17" ht="43.5" spans="2:4">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="17" ht="45" spans="2:4">
       <c r="B17" s="5" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="18" spans="2:6">
       <c r="B18" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D18" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="19" ht="159.5" spans="2:5">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="19" ht="165" spans="2:5">
       <c r="B19" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E19" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="20" spans="2:4">
@@ -10151,7 +10182,7 @@
         <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1" spans="2:4">
@@ -10159,7 +10190,7 @@
         <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D21" s="14"/>
     </row>

</xml_diff>

<commit_message>
fix: update xslt file to change the logic for getting the status of grouper observation resource in the FHIR bundle from HL7 files #2841 - Updated XSLT files to remove unused codes from address.use and telecom.use for all the CCDA and HL7 files - Add the 100698-0 code when NYSAHCHRSN or NYS-AHC-HRSN screening code is provided in the observation grouper resource - Updated the HL7 and CCDA conversion specification documents - Updated Observation Status to correct the mapping in HL7 files - Updated Observation Status to remove preliminary and registered in FHIR Bundle generated from CCDA files since it shows validation error - Updated the CCDA/HL7 to FHIR convertion specification documents
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="9"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="450">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -633,9 +633,8 @@
       </rPr>
       <t xml:space="preserve">
 WP, DIR, PUB -&gt; work
-BA -&gt; billing
 TMP -&gt; temp
-OLD, BAD -&gt; old
+BAD -&gt; old
 All Others -&gt; home</t>
     </r>
   </si>
@@ -727,8 +726,8 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-AS, DIR, PUB, WP, WPN -&gt; work
-H, HP, HV, PRN, ORN, PRS -&gt; home
+AS, DIR, PUB, WP -&gt; work
+H, HP, HV, EC -&gt; home
 MC, PG -&gt; mobile
 TMP -&gt; temp
 BAD -&gt; old
@@ -3848,7 +3847,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-AS, DIR, PUB, WP, WPN -&gt; work
+AS, DIR, PUB, WP -&gt; work
 MC, PG -&gt; mobile
 TMP -&gt; temp
 BAD -&gt; old
@@ -3898,9 +3897,8 @@
       </rPr>
       <t xml:space="preserve">
 WP, DIR, PUB -&gt; work
-BA -&gt; billing
 TMP -&gt; temp
-OLD, BAD -&gt; old
+BAD -&gt; old
 All Others -&gt; work</t>
     </r>
   </si>
@@ -4418,6 +4416,27 @@
   </si>
   <si>
     <t>statusCode.code</t>
+  </si>
+  <si>
+    <r>
+      <t>statusCode.code -&gt; status Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+completed -&gt; final 
+final -&gt; final 
+aborted -&gt; entered-in-error  
+cancelled -&gt; entered-in-error  
+nullified -&gt; entered-in-error 
+All Others -&gt; unknown</t>
+    </r>
   </si>
   <si>
     <t>category</t>
@@ -5683,7 +5702,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5742,6 +5761,23 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10.5"/>
+      <color rgb="FF00B050"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -5917,21 +5953,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color rgb="FF00B050"/>
       <name val="Consolas"/>
@@ -5957,9 +5978,9 @@
       <charset val="134"/>
     </font>
     <font>
-      <i/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF00B050"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5967,7 +5988,22 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6305,137 +6341,137 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6484,19 +6520,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6511,7 +6553,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7074,18 +7116,18 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="30"/>
+    <col min="1" max="1" width="8.88571428571429" style="32"/>
     <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
     <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="30">
+      <c r="A3" s="32">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -7096,7 +7138,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="30">
+      <c r="A4" s="32">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -7107,10 +7149,10 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="30">
+      <c r="A5" s="32">
         <v>3</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="19" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -7118,10 +7160,10 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="30">
+      <c r="A6" s="32">
         <v>4</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="26" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -7129,10 +7171,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="30">
+      <c r="A7" s="32">
         <v>5</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -7184,7 +7226,7 @@
         <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -7195,7 +7237,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="4" ht="60" spans="2:7">
@@ -7206,7 +7248,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -7225,13 +7267,13 @@
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="7" spans="2:6">
@@ -7239,20 +7281,20 @@
         <v>324</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D7" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="90" spans="2:5">
+    <row r="8" customFormat="1" ht="75" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>86</v>
@@ -7266,7 +7308,7 @@
         <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="4"/>
@@ -7276,7 +7318,7 @@
         <v>90</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="4"/>
@@ -7286,7 +7328,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="4"/>
@@ -7296,7 +7338,7 @@
         <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="4"/>
@@ -7306,7 +7348,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="4"/>
@@ -7316,17 +7358,17 @@
         <v>98</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" customFormat="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="4"/>
@@ -7339,7 +7381,7 @@
         <v>193</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
@@ -7349,7 +7391,7 @@
         <v>195</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
@@ -7426,37 +7468,37 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" s="25" customFormat="1" ht="61" customHeight="1" spans="1:4">
-      <c r="A5" s="26"/>
-      <c r="B5" s="26" t="s">
+    <row r="5" s="27" customFormat="1" ht="61" customHeight="1" spans="1:4">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" s="25" customFormat="1" ht="49" customHeight="1" spans="1:4">
-      <c r="A6" s="26"/>
-      <c r="B6" s="26" t="s">
+    <row r="6" s="27" customFormat="1" ht="49" customHeight="1" spans="1:4">
+      <c r="A6" s="28"/>
+      <c r="B6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="27"/>
-    </row>
-    <row r="7" s="25" customFormat="1" ht="86" customHeight="1" spans="1:4">
-      <c r="A7" s="26"/>
-      <c r="B7" s="26" t="s">
+      <c r="D6" s="29"/>
+    </row>
+    <row r="7" s="27" customFormat="1" ht="86" customHeight="1" spans="1:4">
+      <c r="A7" s="28"/>
+      <c r="B7" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="27"/>
+      <c r="D7" s="29"/>
     </row>
     <row r="8" customFormat="1" spans="2:4">
       <c r="B8" t="s">
@@ -7519,7 +7561,7 @@
       <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="18" t="s">
         <v>41</v>
       </c>
     </row>
@@ -7548,7 +7590,7 @@
       <c r="E21" s="8"/>
     </row>
     <row r="22" ht="105" spans="2:3">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="31" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="10" t="s">
@@ -7585,19 +7627,19 @@
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="24" t="s">
         <v>50</v>
       </c>
     </row>
@@ -7754,7 +7796,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" ht="90" spans="2:5">
+    <row r="17" ht="75" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>84</v>
       </c>
@@ -7848,7 +7890,7 @@
       <c r="C26" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="23" t="s">
         <v>107</v>
       </c>
     </row>
@@ -7975,7 +8017,7 @@
         <v>79</v>
       </c>
       <c r="D38" s="14"/>
-      <c r="E38" s="33" t="s">
+      <c r="E38" s="35" t="s">
         <v>129</v>
       </c>
     </row>
@@ -8047,7 +8089,7 @@
       <c r="D45" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="E45" s="16" t="s">
+      <c r="E45" s="18" t="s">
         <v>146</v>
       </c>
     </row>
@@ -8055,7 +8097,7 @@
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="18" t="s">
         <v>148</v>
       </c>
       <c r="D46" s="10" t="s">
@@ -8075,7 +8117,7 @@
       <c r="D47" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E47" s="23"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" customFormat="1" spans="2:5">
       <c r="B48" s="4" t="s">
@@ -8121,7 +8163,7 @@
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="C52" s="16" t="s">
+      <c r="C52" s="18" t="s">
         <v>161</v>
       </c>
       <c r="D52" s="10" t="s">
@@ -8201,7 +8243,7 @@
       <c r="D59" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="E59" s="16" t="s">
+      <c r="E59" s="18" t="s">
         <v>176</v>
       </c>
     </row>
@@ -8392,7 +8434,7 @@
       <c r="C6" t="s">
         <v>201</v>
       </c>
-      <c r="E6" s="24"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" ht="120" spans="2:6">
       <c r="B7" s="5" t="s">
@@ -8501,13 +8543,13 @@
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="18" t="s">
         <v>226</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="18" t="s">
         <v>228</v>
       </c>
     </row>
@@ -8631,7 +8673,7 @@
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="24" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -8705,7 +8747,7 @@
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="18" t="s">
         <v>250</v>
       </c>
       <c r="D7" t="s">
@@ -8735,7 +8777,7 @@
         <v>257</v>
       </c>
       <c r="D9" s="10"/>
-      <c r="E9" s="23"/>
+      <c r="E9" s="25"/>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="5" t="s">
@@ -8751,7 +8793,7 @@
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="18" t="s">
         <v>261</v>
       </c>
       <c r="D11" s="12" t="s">
@@ -8843,7 +8885,7 @@
       <c r="C20" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="E20" s="17"/>
+      <c r="E20" s="19"/>
     </row>
     <row r="21" ht="409.5" spans="2:5">
       <c r="B21" t="s">
@@ -8863,7 +8905,7 @@
       <c r="C22" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="E22" s="20"/>
+      <c r="E22" s="22"/>
     </row>
     <row r="23" ht="66" customHeight="1" spans="2:5">
       <c r="B23" t="s">
@@ -9019,7 +9061,7 @@
       <c r="B8" t="s">
         <v>303</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="18" t="s">
         <v>304</v>
       </c>
       <c r="D8" s="10" t="s">
@@ -9073,7 +9115,7 @@
       <c r="B13" t="s">
         <v>314</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="18" t="s">
         <v>315</v>
       </c>
       <c r="D13" s="10" t="s">
@@ -9091,7 +9133,7 @@
         <v>318</v>
       </c>
       <c r="D14" s="10"/>
-      <c r="E14" s="20"/>
+      <c r="E14" s="22"/>
     </row>
     <row r="15" customFormat="1" ht="30" spans="2:5">
       <c r="B15" s="4" t="s">
@@ -9101,7 +9143,7 @@
         <v>320</v>
       </c>
       <c r="D15" s="10"/>
-      <c r="E15" s="20"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" customFormat="1" ht="30" spans="2:5">
       <c r="B16" s="4" t="s">
@@ -9126,7 +9168,7 @@
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="18" t="s">
         <v>325</v>
       </c>
       <c r="D18" s="10" t="s">
@@ -9188,7 +9230,7 @@
         <v>335</v>
       </c>
       <c r="D23" s="10"/>
-      <c r="E23" s="21" t="s">
+      <c r="E23" s="23" t="s">
         <v>336</v>
       </c>
       <c r="F23" s="4"/>
@@ -9206,7 +9248,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="90" spans="2:6">
+    <row r="25" customFormat="1" ht="75" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
@@ -9343,7 +9385,7 @@
       </c>
     </row>
     <row r="2" ht="45" spans="1:1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>348</v>
       </c>
     </row>
@@ -9527,7 +9569,7 @@
       <c r="D19" t="s">
         <v>376</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="19" t="s">
         <v>377</v>
       </c>
     </row>
@@ -9606,7 +9648,7 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="18"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1"/>
@@ -9622,13 +9664,13 @@
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="18" t="s">
         <v>381</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="E4" s="16"/>
+      <c r="E4" s="18"/>
     </row>
     <row r="5" customFormat="1" spans="1:6">
       <c r="A5" s="1"/>
@@ -9664,7 +9706,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="150" spans="2:5">
+    <row r="8" ht="105" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9674,19 +9716,19 @@
       <c r="D8" t="s">
         <v>354</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>355</v>
+      <c r="E8" s="16" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="9" ht="139" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="E9" s="16" t="s">
         <v>387</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="10" ht="45" spans="2:5">
@@ -9694,11 +9736,11 @@
         <v>219</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" ht="210" spans="2:5">
@@ -9707,7 +9749,7 @@
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="12" ht="210" spans="2:5">
@@ -9716,30 +9758,30 @@
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="5" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1" spans="2:5">
       <c r="B14" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="C14" s="16" t="s">
-        <v>394</v>
+      <c r="C14" s="18" t="s">
+        <v>395</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="E14" s="16" t="s">
-        <v>395</v>
+      <c r="E14" s="18" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="15" spans="2:5">
@@ -9767,11 +9809,11 @@
         <v>362</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="8" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="18" ht="105" spans="2:5">
@@ -9779,13 +9821,13 @@
         <v>363</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="E18" s="16" t="s">
         <v>400</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="19" ht="30" spans="2:3">
@@ -9793,7 +9835,7 @@
         <v>366</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" ht="30" spans="2:3">
@@ -9806,35 +9848,35 @@
     </row>
     <row r="21" ht="37" customHeight="1" spans="2:5">
       <c r="B21" s="5" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E21" s="8"/>
     </row>
     <row r="22" ht="75" spans="2:5">
       <c r="B22" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C22" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="11" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="23" ht="45" spans="2:5">
       <c r="B23" s="5" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="24" ht="75" spans="2:4">
@@ -9858,13 +9900,13 @@
     </row>
     <row r="26" ht="45" spans="2:4">
       <c r="B26" s="5" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C26" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="27" ht="210" spans="2:5">
@@ -9875,19 +9917,19 @@
       <c r="D27" t="s">
         <v>373</v>
       </c>
-      <c r="E27" s="16" t="s">
-        <v>413</v>
+      <c r="E27" s="18" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="28" ht="45" spans="2:4">
       <c r="B28" s="5" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="29" spans="2:6">
@@ -9910,7 +9952,7 @@
         <v>193</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="31" ht="46" customHeight="1" spans="2:4">
@@ -9974,7 +10016,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9999,7 +10041,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -10033,13 +10075,13 @@
         <v>57</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="150" spans="2:5">
+    <row r="8" ht="105" spans="2:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -10049,19 +10091,20 @@
       <c r="D8" t="s">
         <v>354</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>355</v>
-      </c>
+      <c r="E8" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="F8" s="17"/>
     </row>
     <row r="9" ht="409" customHeight="1" spans="2:5">
       <c r="B9" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="10" ht="165" spans="2:5">
@@ -10072,10 +10115,10 @@
         <v>254</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="E10" s="16" t="s">
         <v>423</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="11" ht="180" spans="2:5">
@@ -10084,7 +10127,7 @@
       </c>
       <c r="C11" s="4"/>
       <c r="E11" s="11" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="12" ht="150" spans="2:5">
@@ -10093,7 +10136,7 @@
       </c>
       <c r="C12" s="4"/>
       <c r="E12" s="11" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="13" ht="75" spans="2:4">
@@ -10117,13 +10160,13 @@
     </row>
     <row r="15" ht="45" spans="2:4">
       <c r="B15" s="5" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="16" ht="210" spans="2:5">
@@ -10134,19 +10177,19 @@
       <c r="D16" t="s">
         <v>373</v>
       </c>
-      <c r="E16" s="16" t="s">
-        <v>413</v>
+      <c r="E16" s="18" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="17" ht="45" spans="2:4">
       <c r="B17" s="5" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" spans="2:6">
@@ -10157,21 +10200,21 @@
         <v>376</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>426</v>
-      </c>
-      <c r="F18" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="19" ht="165" spans="2:5">
       <c r="B19" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E19" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="20" spans="2:4">
@@ -10182,7 +10225,7 @@
         <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1" spans="2:4">

</xml_diff>

<commit_message>
fix: update system value for screening codes in HL7 grouper observation resources #2841 - Updated the system for screening codes NYSAHCHRSN and NYS-AHC-HRSN to base_url/CodeSystem/NYS-HRSN-Questionnaire and for 96777-8, 97023-6 and 100698-0 as http://loinc.org in grouper observation resource - Removed space from address and telecom 'use' value before assigning the mapping values. - Updated the CCDA/Hl7 to FHIR conversion specification documents
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="7"/>
+    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="451">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -612,15 +612,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>addr.use -&gt; use Mapping</t>
     </r>
     <r>
@@ -635,7 +626,7 @@
 WP, DIR, PUB -&gt; work
 TMP -&gt; temp
 BAD -&gt; old
-All Others -&gt; home</t>
+All Others (H, HP, HV, AS, EC, MC, PG) -&gt; home</t>
     </r>
   </si>
   <si>
@@ -706,15 +697,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>telecom -&gt; use Mapping</t>
     </r>
     <r>
@@ -730,8 +712,7 @@
 H, HP, HV, EC -&gt; home
 MC, PG -&gt; mobile
 TMP -&gt; temp
-BAD -&gt; old
-All others -&gt; home</t>
+BAD -&gt; old</t>
     </r>
   </si>
   <si>
@@ -3827,15 +3808,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>telecom -&gt; use Mapping</t>
     </r>
     <r>
@@ -3851,7 +3823,7 @@
 MC, PG -&gt; mobile
 TMP -&gt; temp
 BAD -&gt; old
-All others -&gt; work</t>
+All others (H, HP, HV, EC) -&gt; work</t>
     </r>
   </si>
   <si>
@@ -3876,15 +3848,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>addr.use -&gt; use Mapping</t>
     </r>
     <r>
@@ -3899,7 +3862,7 @@
 WP, DIR, PUB -&gt; work
 TMP -&gt; temp
 BAD -&gt; old
-All Others -&gt; work</t>
+All Others (H, HP, HV, AS, EC, MC, PG) -&gt; work</t>
     </r>
   </si>
   <si>
@@ -4419,6 +4382,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>statusCode.code -&gt; status Mapping</t>
     </r>
     <r>
@@ -5654,6 +5626,25 @@
   </si>
   <si>
     <t>addr.use</t>
+  </si>
+  <si>
+    <r>
+      <t>addr.use -&gt; use Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+WP, DIR, PUB -&gt; work
+TMP -&gt; temp
+BAD -&gt; old
+All Others (H, HP, HV, AS, EC, MC, PG, BA) -&gt; work</t>
+    </r>
   </si>
   <si>
     <t>addr.streetAddressLine
@@ -5953,6 +5944,37 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <color rgb="FF00B050"/>
       <name val="Consolas"/>
@@ -5976,37 +5998,6 @@
       <color rgb="FF00B050"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -7114,11 +7105,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="32"/>
-    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
-    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="8.88181818181818" style="32"/>
+    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
+    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
@@ -7191,14 +7182,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7240,7 +7231,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="4" ht="60" spans="2:7">
+    <row r="4" ht="58" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7262,7 +7253,7 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="29" spans="2:6">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -7289,7 +7280,7 @@
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="75" spans="2:5">
+    <row r="8" customFormat="1" ht="72.5" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
@@ -7300,15 +7291,15 @@
         <v>86</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" ht="60" spans="2:5">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="58" spans="2:5">
       <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="4"/>
@@ -7318,7 +7309,7 @@
         <v>90</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="4"/>
@@ -7328,7 +7319,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="4"/>
@@ -7338,7 +7329,7 @@
         <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="4"/>
@@ -7348,7 +7339,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="4"/>
@@ -7358,17 +7349,17 @@
         <v>98</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="4"/>
     </row>
     <row r="15" customFormat="1" spans="2:5">
       <c r="B15" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="4"/>
@@ -7381,7 +7372,7 @@
         <v>193</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
@@ -7391,7 +7382,7 @@
         <v>195</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
@@ -7412,14 +7403,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
-    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
+    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7517,7 +7508,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="30" spans="2:3">
+    <row r="10" customFormat="1" ht="29" spans="2:3">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7538,7 +7529,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="2:3">
+    <row r="16" ht="72.5" spans="2:3">
       <c r="B16" t="s">
         <v>35</v>
       </c>
@@ -7554,7 +7545,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="75" spans="2:5">
+    <row r="18" ht="72.5" spans="2:5">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -7565,7 +7556,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="45" spans="2:5">
+    <row r="19" ht="29" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
@@ -7574,7 +7565,7 @@
       </c>
       <c r="E19" s="10"/>
     </row>
-    <row r="20" ht="45" spans="2:5">
+    <row r="20" ht="43.5" spans="2:5">
       <c r="B20" t="s">
         <v>44</v>
       </c>
@@ -7583,13 +7574,13 @@
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="30" spans="2:5">
+    <row r="21" ht="29" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="105" spans="2:3">
+    <row r="22" ht="101.5" spans="2:3">
       <c r="B22" s="31" t="s">
         <v>47</v>
       </c>
@@ -7613,13 +7604,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7685,7 +7676,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="30" spans="2:4">
+    <row r="7" ht="29" spans="2:4">
       <c r="B7" s="4" t="s">
         <v>55</v>
       </c>
@@ -7696,7 +7687,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" ht="60" spans="2:5">
+    <row r="8" ht="58" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
@@ -7752,7 +7743,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" ht="60" spans="2:4">
+    <row r="13" ht="58" spans="2:4">
       <c r="B13" s="4" t="s">
         <v>72</v>
       </c>
@@ -7763,7 +7754,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="2:4">
+    <row r="14" ht="29" spans="2:4">
       <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
@@ -7774,7 +7765,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" ht="30" spans="2:4">
+    <row r="15" ht="29" spans="2:4">
       <c r="B15" s="4" t="s">
         <v>78</v>
       </c>
@@ -7796,7 +7787,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" ht="75" spans="2:5">
+    <row r="17" ht="72.5" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>84</v>
       </c>
@@ -7810,7 +7801,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="60" spans="2:4">
+    <row r="18" ht="58" spans="2:4">
       <c r="B18" s="4" t="s">
         <v>88</v>
       </c>
@@ -7883,7 +7874,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="26" ht="105" spans="2:5">
+    <row r="26" ht="87" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>105</v>
       </c>
@@ -7894,7 +7885,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" ht="45" spans="2:5">
+    <row r="27" ht="43.5" spans="2:5">
       <c r="B27" s="4" t="s">
         <v>108</v>
       </c>
@@ -7908,7 +7899,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" ht="30" spans="2:5">
+    <row r="28" spans="2:5">
       <c r="B28" s="4" t="s">
         <v>112</v>
       </c>
@@ -7928,7 +7919,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" ht="30" spans="2:5">
+    <row r="30" spans="2:5">
       <c r="B30" s="4" t="s">
         <v>116</v>
       </c>
@@ -7948,7 +7939,7 @@
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" ht="45" spans="2:5">
+    <row r="32" ht="43.5" spans="2:5">
       <c r="B32" s="4" t="s">
         <v>108</v>
       </c>
@@ -7962,7 +7953,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" ht="30" spans="2:4">
+    <row r="33" spans="2:4">
       <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
@@ -7980,7 +7971,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" ht="30" spans="2:4">
+    <row r="35" spans="2:4">
       <c r="B35" s="4" t="s">
         <v>116</v>
       </c>
@@ -8009,7 +8000,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" ht="45" spans="2:5">
+    <row r="38" ht="43.5" spans="2:5">
       <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
@@ -8021,7 +8012,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" ht="120" spans="2:6">
+    <row r="39" ht="116" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>130</v>
       </c>
@@ -8032,7 +8023,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" ht="120" spans="2:6">
+    <row r="40" ht="116" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>133</v>
       </c>
@@ -8079,7 +8070,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="195" spans="2:5">
+    <row r="45" ht="188.5" spans="2:5">
       <c r="B45" s="15" t="s">
         <v>143</v>
       </c>
@@ -8093,7 +8084,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" ht="195" spans="2:5">
+    <row r="46" ht="188.5" spans="2:5">
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
@@ -8107,7 +8098,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" ht="195" spans="2:5">
+    <row r="47" ht="188.5" spans="2:5">
       <c r="B47" s="15" t="s">
         <v>151</v>
       </c>
@@ -8159,7 +8150,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="150" spans="2:5">
+    <row r="52" ht="145" spans="2:5">
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
@@ -8233,7 +8224,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="180" spans="2:5">
+    <row r="59" ht="174" spans="2:5">
       <c r="B59" s="10" t="s">
         <v>174</v>
       </c>
@@ -8247,7 +8238,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="60" ht="255" spans="2:6">
+    <row r="60" ht="246.5" spans="2:6">
       <c r="B60" s="4" t="s">
         <v>177</v>
       </c>
@@ -8278,7 +8269,7 @@
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="210" spans="2:6">
+    <row r="63" ht="203" spans="2:6">
       <c r="B63" s="4" t="s">
         <v>184</v>
       </c>
@@ -8356,14 +8347,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8405,7 +8396,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" ht="60" spans="2:7">
+    <row r="4" ht="58" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8436,7 +8427,7 @@
       </c>
       <c r="E6" s="26"/>
     </row>
-    <row r="7" ht="120" spans="2:6">
+    <row r="7" ht="116" spans="2:6">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8489,7 +8480,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" ht="225" spans="2:5">
+    <row r="11" ht="203" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -8525,7 +8516,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" ht="45" spans="2:5">
+    <row r="14" ht="43.5" spans="2:5">
       <c r="B14" s="5" t="s">
         <v>221</v>
       </c>
@@ -8539,7 +8530,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" ht="255" spans="2:5">
+    <row r="15" ht="246.5" spans="2:5">
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
@@ -8553,7 +8544,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" ht="45" spans="2:5">
+    <row r="16" ht="43.5" spans="2:5">
       <c r="B16" s="5" t="s">
         <v>229</v>
       </c>
@@ -8565,7 +8556,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="45" spans="2:5">
+    <row r="17" ht="43.5" spans="2:5">
       <c r="B17" s="5" t="s">
         <v>232</v>
       </c>
@@ -8577,7 +8568,7 @@
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="45" spans="2:5">
+    <row r="18" ht="43.5" spans="2:5">
       <c r="B18" t="s">
         <v>235</v>
       </c>
@@ -8591,7 +8582,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="60" spans="2:5">
+    <row r="19" ht="58" spans="2:5">
       <c r="B19" s="5" t="s">
         <v>238</v>
       </c>
@@ -8656,14 +8647,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="42.2857142857143" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
+    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8705,7 +8696,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" ht="75" spans="1:5">
+    <row r="4" ht="72.5" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8732,7 +8723,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -8743,7 +8734,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="255" spans="2:5">
+    <row r="7" ht="246.5" spans="2:5">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8769,7 +8760,7 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="30" spans="2:5">
+    <row r="9" ht="29" spans="2:5">
       <c r="B9" s="5" t="s">
         <v>256</v>
       </c>
@@ -8789,7 +8780,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="30" spans="2:4">
+    <row r="11" ht="29" spans="2:4">
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
@@ -8800,7 +8791,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" ht="60" spans="2:5">
+    <row r="12" ht="58" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>263</v>
       </c>
@@ -8826,7 +8817,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="60" spans="2:4">
+    <row r="15" customFormat="1" ht="58" spans="2:4">
       <c r="B15" s="5" t="s">
         <v>269</v>
       </c>
@@ -8837,7 +8828,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="2:3">
+    <row r="16" customFormat="1" ht="29" spans="2:3">
       <c r="B16" s="5" t="s">
         <v>271</v>
       </c>
@@ -8845,7 +8836,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" ht="60" spans="2:4">
+    <row r="17" ht="58" spans="2:4">
       <c r="B17" t="s">
         <v>273</v>
       </c>
@@ -8864,7 +8855,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" ht="45" spans="2:5">
+    <row r="19" ht="43.5" spans="2:5">
       <c r="B19" t="s">
         <v>278</v>
       </c>
@@ -8898,7 +8889,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="22" ht="60" spans="2:5">
+    <row r="22" ht="58" spans="2:5">
       <c r="B22" t="s">
         <v>287</v>
       </c>
@@ -8967,14 +8958,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
-    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
+    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9032,7 +9023,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -9081,7 +9072,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="30" spans="2:5">
+    <row r="10" ht="29" spans="2:5">
       <c r="B10" s="4" t="s">
         <v>309</v>
       </c>
@@ -9091,7 +9082,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="30" spans="2:5">
+    <row r="11" ht="29" spans="2:5">
       <c r="B11" s="4" t="s">
         <v>311</v>
       </c>
@@ -9101,7 +9092,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:5">
+    <row r="12" ht="29" spans="2:5">
       <c r="B12" s="4" t="s">
         <v>312</v>
       </c>
@@ -9135,7 +9126,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" customFormat="1" ht="30" spans="2:5">
+    <row r="15" customFormat="1" ht="29" spans="2:5">
       <c r="B15" s="4" t="s">
         <v>319</v>
       </c>
@@ -9145,7 +9136,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="22"/>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="2:5">
+    <row r="16" customFormat="1" ht="29" spans="2:5">
       <c r="B16" s="4" t="s">
         <v>321</v>
       </c>
@@ -9155,7 +9146,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="30" spans="2:4">
+    <row r="17" customFormat="1" ht="29" spans="2:4">
       <c r="B17" s="4" t="s">
         <v>322</v>
       </c>
@@ -9164,7 +9155,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="60" spans="2:5">
+    <row r="18" ht="58" spans="2:5">
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
@@ -9212,7 +9203,7 @@
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="30" spans="2:6">
+    <row r="22" customFormat="1" ht="29" spans="2:6">
       <c r="B22" s="4" t="s">
         <v>103</v>
       </c>
@@ -9222,7 +9213,7 @@
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="90" spans="2:6">
+    <row r="23" customFormat="1" ht="87" spans="2:6">
       <c r="B23" s="4" t="s">
         <v>105</v>
       </c>
@@ -9235,7 +9226,7 @@
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="120" spans="2:6">
+    <row r="24" customFormat="1" ht="116" spans="2:6">
       <c r="B24" s="4" t="s">
         <v>88</v>
       </c>
@@ -9248,7 +9239,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="75" spans="2:6">
+    <row r="25" customFormat="1" ht="72.5" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
@@ -9261,7 +9252,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="30" spans="2:6">
+    <row r="26" customFormat="1" ht="29" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>90</v>
       </c>
@@ -9272,7 +9263,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="30" spans="2:6">
+    <row r="27" customFormat="1" ht="29" spans="2:6">
       <c r="B27" s="4" t="s">
         <v>92</v>
       </c>
@@ -9283,7 +9274,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="30" spans="2:6">
+    <row r="28" customFormat="1" ht="29" spans="2:6">
       <c r="B28" s="4" t="s">
         <v>94</v>
       </c>
@@ -9294,7 +9285,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="30" spans="2:6">
+    <row r="29" customFormat="1" ht="29" spans="2:6">
       <c r="B29" s="4" t="s">
         <v>96</v>
       </c>
@@ -9305,7 +9296,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="30" spans="2:6">
+    <row r="30" customFormat="1" ht="29" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>98</v>
       </c>
@@ -9354,13 +9345,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="46.8571428571429" customWidth="1"/>
-    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
-    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
+    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
+    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9384,7 +9375,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="45" spans="1:1">
+    <row r="2" ht="43.5" spans="1:1">
       <c r="A2" s="21" t="s">
         <v>348</v>
       </c>
@@ -9422,7 +9413,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9444,7 +9435,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="150" spans="2:5">
+    <row r="8" ht="145" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9469,7 +9460,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="10" ht="30" spans="2:4">
+    <row r="10" ht="29" spans="2:4">
       <c r="B10" s="5" t="s">
         <v>359</v>
       </c>
@@ -9488,7 +9479,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:4">
+    <row r="12" ht="29" spans="2:4">
       <c r="B12" s="5" t="s">
         <v>362</v>
       </c>
@@ -9508,7 +9499,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="2:4">
+    <row r="14" ht="29" spans="2:4">
       <c r="B14" s="4" t="s">
         <v>366</v>
       </c>
@@ -9529,7 +9520,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="2:4">
+    <row r="16" ht="58" spans="2:4">
       <c r="B16" s="5" t="s">
         <v>269</v>
       </c>
@@ -9540,7 +9531,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" ht="30" spans="2:3">
+    <row r="17" ht="29" spans="2:3">
       <c r="B17" s="5" t="s">
         <v>271</v>
       </c>
@@ -9548,7 +9539,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="18" ht="90" spans="2:5">
+    <row r="18" ht="87" spans="2:5">
       <c r="B18" t="s">
         <v>371</v>
       </c>
@@ -9608,14 +9599,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9659,7 +9650,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="4" ht="78" spans="1:5">
+    <row r="4" ht="82.5" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -9684,7 +9675,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9706,7 +9697,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="2:5">
+    <row r="8" ht="101.5" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9731,7 +9722,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="10" ht="45" spans="2:5">
+    <row r="10" ht="43.5" spans="2:5">
       <c r="B10" s="5" t="s">
         <v>219</v>
       </c>
@@ -9743,7 +9734,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="11" ht="210" spans="2:5">
+    <row r="11" ht="203" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -9752,7 +9743,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="12" ht="210" spans="2:5">
+    <row r="12" ht="203" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
@@ -9804,7 +9795,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="30" spans="2:5">
+    <row r="17" ht="29" spans="2:5">
       <c r="B17" s="5" t="s">
         <v>362</v>
       </c>
@@ -9816,7 +9807,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="18" ht="105" spans="2:5">
+    <row r="18" ht="101.5" spans="2:5">
       <c r="B18" s="4" t="s">
         <v>363</v>
       </c>
@@ -9830,7 +9821,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="19" ht="30" spans="2:3">
+    <row r="19" ht="29" spans="2:3">
       <c r="B19" s="4" t="s">
         <v>366</v>
       </c>
@@ -9838,7 +9829,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="20" ht="30" spans="2:3">
+    <row r="20" ht="29" spans="2:3">
       <c r="B20" s="4" t="s">
         <v>368</v>
       </c>
@@ -9858,7 +9849,7 @@
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="75" spans="2:5">
+    <row r="22" ht="72.5" spans="2:5">
       <c r="B22" s="5" t="s">
         <v>406</v>
       </c>
@@ -9870,7 +9861,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="23" ht="45" spans="2:5">
+    <row r="23" ht="43.5" spans="2:5">
       <c r="B23" s="5" t="s">
         <v>409</v>
       </c>
@@ -9879,7 +9870,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="24" ht="75" spans="2:4">
+    <row r="24" ht="58" spans="2:4">
       <c r="B24" s="5" t="s">
         <v>269</v>
       </c>
@@ -9890,7 +9881,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" ht="30" spans="2:3">
+    <row r="25" ht="29" spans="2:3">
       <c r="B25" s="5" t="s">
         <v>271</v>
       </c>
@@ -9898,7 +9889,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="26" ht="45" spans="2:4">
+    <row r="26" ht="43.5" spans="2:4">
       <c r="B26" s="5" t="s">
         <v>411</v>
       </c>
@@ -9909,7 +9900,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="27" ht="210" spans="2:5">
+    <row r="27" ht="203" spans="2:5">
       <c r="B27" s="5" t="s">
         <v>371</v>
       </c>
@@ -9921,7 +9912,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="28" ht="45" spans="2:4">
+    <row r="28" ht="43.5" spans="2:4">
       <c r="B28" s="5" t="s">
         <v>415</v>
       </c>
@@ -9981,14 +9972,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -10056,7 +10047,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="29" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -10081,7 +10072,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="2:6">
+    <row r="8" ht="101.5" spans="2:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -10107,7 +10098,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="10" ht="165" spans="2:5">
+    <row r="10" ht="159.5" spans="2:5">
       <c r="B10" s="5" t="s">
         <v>356</v>
       </c>
@@ -10121,7 +10112,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="11" ht="180" spans="2:5">
+    <row r="11" ht="159.5" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>359</v>
       </c>
@@ -10130,7 +10121,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="12" ht="150" spans="2:5">
+    <row r="12" ht="145" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>361</v>
       </c>
@@ -10139,7 +10130,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="13" ht="75" spans="2:4">
+    <row r="13" ht="58" spans="2:4">
       <c r="B13" s="5" t="s">
         <v>269</v>
       </c>
@@ -10150,7 +10141,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="2:3">
+    <row r="14" ht="29" spans="2:3">
       <c r="B14" s="5" t="s">
         <v>271</v>
       </c>
@@ -10158,7 +10149,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" ht="45" spans="2:4">
+    <row r="15" ht="43.5" spans="2:4">
       <c r="B15" s="5" t="s">
         <v>411</v>
       </c>
@@ -10169,7 +10160,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="16" ht="210" spans="2:5">
+    <row r="16" ht="203" spans="2:5">
       <c r="B16" s="5" t="s">
         <v>371</v>
       </c>
@@ -10181,7 +10172,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="17" ht="45" spans="2:4">
+    <row r="17" ht="43.5" spans="2:4">
       <c r="B17" s="5" t="s">
         <v>415</v>
       </c>
@@ -10206,7 +10197,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="19" ht="165" spans="2:5">
+    <row r="19" ht="159.5" spans="2:5">
       <c r="B19" t="s">
         <v>428</v>
       </c>

</xml_diff>

<commit_message>
feat: update CCDA-to-FHIR Conversion XSLT Files to consolidate common logic and apply vendor updates #2909 - incorporated the recent updates made to the Epic, Medent, and AthenaHealth CCDA-to-FHIR conversion XSLT files into the generic XSLT used for processing CCDA files from other vendors. - added a common utility XSLT file and moved all reusable functions and templates into this common file. - updated all the vendor-specific and generic XSLT files to reference the common utility XSLT file. - updated telecom.system mapping in HL7 and CCDA files. - updated the CCDA and HL7 to FHIR conversion specification documents with the telecom.system mapping.
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -612,6 +612,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>addr.use -&gt; use Mapping</t>
     </r>
     <r>
@@ -679,9 +688,37 @@
       }],</t>
   </si>
   <si>
-    <t>If telecom.value contains "tel:" then "phone".
-If telecom.value contains "mailto:" then "email".
-Otherwise "other"</t>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>telecom.value</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> contains 
+  "tel:" then "phone",
+  "mailto:" then "email",
+  "fax:" then "fax",
+  "pager:" then "pager",
+  "sms:" then "sms",
+  "http://" or "https://" or "www." then "url",
+  All Others "other".</t>
+    </r>
   </si>
   <si>
     <t>telecom -&gt; value</t>
@@ -697,6 +734,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>telecom -&gt; use Mapping</t>
     </r>
     <r>
@@ -3808,6 +3854,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>telecom -&gt; use Mapping</t>
     </r>
     <r>
@@ -3848,6 +3903,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>addr.use -&gt; use Mapping</t>
     </r>
     <r>
@@ -5629,6 +5693,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>addr.use -&gt; use Mapping</t>
     </r>
     <r>
@@ -5958,22 +6031,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF00B050"/>
@@ -5998,6 +6055,22 @@
       <color rgb="FF00B050"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -7105,11 +7178,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88181818181818" style="32"/>
-    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
-    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
+    <col min="1" max="1" width="8.88571428571429" style="32"/>
+    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
+    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
@@ -7182,14 +7255,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7231,7 +7304,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="4" ht="58" spans="2:7">
+    <row r="4" ht="60" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7253,7 +7326,7 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="29" spans="2:6">
+    <row r="6" ht="30" spans="2:6">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -7280,7 +7353,7 @@
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="72.5" spans="2:5">
+    <row r="8" customFormat="1" ht="75" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
@@ -7294,7 +7367,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="9" customFormat="1" ht="58" spans="2:5">
+    <row r="9" customFormat="1" ht="60" spans="2:5">
       <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
@@ -7403,14 +7476,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="65.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
-    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="65.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
+    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7508,7 +7581,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="29" spans="2:3">
+    <row r="10" customFormat="1" ht="30" spans="2:3">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7529,7 +7602,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="72.5" spans="2:3">
+    <row r="16" ht="75" spans="2:3">
       <c r="B16" t="s">
         <v>35</v>
       </c>
@@ -7545,7 +7618,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="72.5" spans="2:5">
+    <row r="18" ht="75" spans="2:5">
       <c r="B18" t="s">
         <v>39</v>
       </c>
@@ -7556,7 +7629,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" ht="29" spans="2:5">
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>42</v>
       </c>
@@ -7565,7 +7638,7 @@
       </c>
       <c r="E19" s="10"/>
     </row>
-    <row r="20" ht="43.5" spans="2:5">
+    <row r="20" ht="45" spans="2:5">
       <c r="B20" t="s">
         <v>44</v>
       </c>
@@ -7574,13 +7647,13 @@
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="29" spans="2:5">
+    <row r="21" ht="30" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>46</v>
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="101.5" spans="2:3">
+    <row r="22" ht="105" spans="2:3">
       <c r="B22" s="31" t="s">
         <v>47</v>
       </c>
@@ -7604,13 +7677,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
-    <col min="3" max="3" width="63.8818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
+    <col min="3" max="3" width="63.8857142857143" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7676,7 +7749,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="29" spans="2:4">
+    <row r="7" ht="30" spans="2:4">
       <c r="B7" s="4" t="s">
         <v>55</v>
       </c>
@@ -7687,7 +7760,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" ht="58" spans="2:5">
+    <row r="8" ht="60" spans="2:5">
       <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
@@ -7743,7 +7816,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" ht="58" spans="2:4">
+    <row r="13" ht="60" spans="2:4">
       <c r="B13" s="4" t="s">
         <v>72</v>
       </c>
@@ -7754,7 +7827,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" ht="29" spans="2:4">
+    <row r="14" ht="30" spans="2:4">
       <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
@@ -7765,7 +7838,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" ht="29" spans="2:4">
+    <row r="15" ht="30" spans="2:4">
       <c r="B15" s="4" t="s">
         <v>78</v>
       </c>
@@ -7787,7 +7860,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" ht="72.5" spans="2:5">
+    <row r="17" ht="75" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>84</v>
       </c>
@@ -7801,7 +7874,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="58" spans="2:4">
+    <row r="18" ht="60" spans="2:4">
       <c r="B18" s="4" t="s">
         <v>88</v>
       </c>
@@ -7855,14 +7928,14 @@
       </c>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" ht="48" customHeight="1" spans="2:5">
+    <row r="24" ht="120" spans="2:5">
       <c r="B24" s="4" t="s">
         <v>100</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="18" t="s">
         <v>102</v>
       </c>
     </row>
@@ -7874,7 +7947,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="26" ht="87" spans="2:5">
+    <row r="26" ht="90" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>105</v>
       </c>
@@ -7885,7 +7958,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" ht="43.5" spans="2:5">
+    <row r="27" ht="45" spans="2:5">
       <c r="B27" s="4" t="s">
         <v>108</v>
       </c>
@@ -7899,7 +7972,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="2:5">
+    <row r="28" ht="30" spans="2:5">
       <c r="B28" s="4" t="s">
         <v>112</v>
       </c>
@@ -7919,7 +7992,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="8"/>
     </row>
-    <row r="30" spans="2:5">
+    <row r="30" ht="30" spans="2:5">
       <c r="B30" s="4" t="s">
         <v>116</v>
       </c>
@@ -7939,7 +8012,7 @@
       <c r="D31" s="14"/>
       <c r="E31" s="8"/>
     </row>
-    <row r="32" ht="43.5" spans="2:5">
+    <row r="32" ht="45" spans="2:5">
       <c r="B32" s="4" t="s">
         <v>108</v>
       </c>
@@ -7953,7 +8026,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="2:4">
+    <row r="33" ht="30" spans="2:4">
       <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
@@ -7971,7 +8044,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" spans="2:4">
+    <row r="35" ht="30" spans="2:4">
       <c r="B35" s="4" t="s">
         <v>116</v>
       </c>
@@ -8000,7 +8073,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" ht="43.5" spans="2:5">
+    <row r="38" ht="45" spans="2:5">
       <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
@@ -8012,7 +8085,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" ht="116" spans="2:6">
+    <row r="39" ht="120" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>130</v>
       </c>
@@ -8023,7 +8096,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" ht="116" spans="2:6">
+    <row r="40" ht="120" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>133</v>
       </c>
@@ -8070,7 +8143,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="188.5" spans="2:5">
+    <row r="45" ht="195" spans="2:5">
       <c r="B45" s="15" t="s">
         <v>143</v>
       </c>
@@ -8084,7 +8157,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" ht="188.5" spans="2:5">
+    <row r="46" ht="195" spans="2:5">
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
@@ -8098,7 +8171,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" ht="188.5" spans="2:5">
+    <row r="47" ht="195" spans="2:5">
       <c r="B47" s="15" t="s">
         <v>151</v>
       </c>
@@ -8150,7 +8223,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="145" spans="2:5">
+    <row r="52" ht="150" spans="2:5">
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
@@ -8224,7 +8297,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="174" spans="2:5">
+    <row r="59" ht="180" spans="2:5">
       <c r="B59" s="10" t="s">
         <v>174</v>
       </c>
@@ -8238,7 +8311,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="60" ht="246.5" spans="2:6">
+    <row r="60" ht="255" spans="2:6">
       <c r="B60" s="4" t="s">
         <v>177</v>
       </c>
@@ -8269,7 +8342,7 @@
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="203" spans="2:6">
+    <row r="63" ht="210" spans="2:6">
       <c r="B63" s="4" t="s">
         <v>184</v>
       </c>
@@ -8347,14 +8420,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
-    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8396,7 +8469,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" ht="58" spans="2:7">
+    <row r="4" ht="60" spans="2:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8427,7 +8500,7 @@
       </c>
       <c r="E6" s="26"/>
     </row>
-    <row r="7" ht="116" spans="2:6">
+    <row r="7" ht="120" spans="2:6">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8480,7 +8553,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" ht="203" spans="2:5">
+    <row r="11" ht="225" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -8516,7 +8589,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" ht="43.5" spans="2:5">
+    <row r="14" ht="45" spans="2:5">
       <c r="B14" s="5" t="s">
         <v>221</v>
       </c>
@@ -8530,7 +8603,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" ht="246.5" spans="2:5">
+    <row r="15" ht="255" spans="2:5">
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
@@ -8544,7 +8617,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" ht="43.5" spans="2:5">
+    <row r="16" ht="45" spans="2:5">
       <c r="B16" s="5" t="s">
         <v>229</v>
       </c>
@@ -8556,7 +8629,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="43.5" spans="2:5">
+    <row r="17" ht="45" spans="2:5">
       <c r="B17" s="5" t="s">
         <v>232</v>
       </c>
@@ -8568,7 +8641,7 @@
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="43.5" spans="2:5">
+    <row r="18" ht="45" spans="2:5">
       <c r="B18" t="s">
         <v>235</v>
       </c>
@@ -8582,7 +8655,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="58" spans="2:5">
+    <row r="19" ht="60" spans="2:5">
       <c r="B19" s="5" t="s">
         <v>238</v>
       </c>
@@ -8647,14 +8720,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
-    <col min="3" max="3" width="42.2818181818182" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="42.2857142857143" style="4" customWidth="1"/>
+    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
+    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8696,7 +8769,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" ht="72.5" spans="1:5">
+    <row r="4" ht="75" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8723,7 +8796,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -8734,7 +8807,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="246.5" spans="2:5">
+    <row r="7" ht="255" spans="2:5">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8760,7 +8833,7 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="29" spans="2:5">
+    <row r="9" ht="30" spans="2:5">
       <c r="B9" s="5" t="s">
         <v>256</v>
       </c>
@@ -8780,7 +8853,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="29" spans="2:4">
+    <row r="11" ht="30" spans="2:4">
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
@@ -8791,7 +8864,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" ht="58" spans="2:5">
+    <row r="12" ht="60" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>263</v>
       </c>
@@ -8817,7 +8890,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="58" spans="2:4">
+    <row r="15" customFormat="1" ht="60" spans="2:4">
       <c r="B15" s="5" t="s">
         <v>269</v>
       </c>
@@ -8828,7 +8901,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="29" spans="2:3">
+    <row r="16" customFormat="1" ht="30" spans="2:3">
       <c r="B16" s="5" t="s">
         <v>271</v>
       </c>
@@ -8836,7 +8909,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" ht="58" spans="2:4">
+    <row r="17" ht="60" spans="2:4">
       <c r="B17" t="s">
         <v>273</v>
       </c>
@@ -8855,7 +8928,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" ht="43.5" spans="2:5">
+    <row r="19" ht="45" spans="2:5">
       <c r="B19" t="s">
         <v>278</v>
       </c>
@@ -8889,7 +8962,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="22" ht="58" spans="2:5">
+    <row r="22" ht="60" spans="2:5">
       <c r="B22" t="s">
         <v>287</v>
       </c>
@@ -8958,14 +9031,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
-    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
-    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
+    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9023,7 +9096,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -9072,7 +9145,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="29" spans="2:5">
+    <row r="10" ht="30" spans="2:5">
       <c r="B10" s="4" t="s">
         <v>309</v>
       </c>
@@ -9082,7 +9155,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="29" spans="2:5">
+    <row r="11" ht="30" spans="2:5">
       <c r="B11" s="4" t="s">
         <v>311</v>
       </c>
@@ -9092,7 +9165,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="29" spans="2:5">
+    <row r="12" ht="30" spans="2:5">
       <c r="B12" s="4" t="s">
         <v>312</v>
       </c>
@@ -9126,7 +9199,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" customFormat="1" ht="29" spans="2:5">
+    <row r="15" customFormat="1" ht="30" spans="2:5">
       <c r="B15" s="4" t="s">
         <v>319</v>
       </c>
@@ -9136,7 +9209,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="22"/>
     </row>
-    <row r="16" customFormat="1" ht="29" spans="2:5">
+    <row r="16" customFormat="1" ht="30" spans="2:5">
       <c r="B16" s="4" t="s">
         <v>321</v>
       </c>
@@ -9146,7 +9219,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="29" spans="2:4">
+    <row r="17" customFormat="1" ht="30" spans="2:4">
       <c r="B17" s="4" t="s">
         <v>322</v>
       </c>
@@ -9155,7 +9228,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="58" spans="2:5">
+    <row r="18" ht="60" spans="2:5">
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
@@ -9190,7 +9263,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="21" customFormat="1" ht="50" customHeight="1" spans="2:6">
+    <row r="21" customFormat="1" ht="120" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>100</v>
       </c>
@@ -9198,12 +9271,12 @@
       <c r="D21" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="18" t="s">
         <v>102</v>
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="29" spans="2:6">
+    <row r="22" customFormat="1" ht="30" spans="2:6">
       <c r="B22" s="4" t="s">
         <v>103</v>
       </c>
@@ -9213,7 +9286,7 @@
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="87" spans="2:6">
+    <row r="23" customFormat="1" ht="90" spans="2:6">
       <c r="B23" s="4" t="s">
         <v>105</v>
       </c>
@@ -9226,7 +9299,7 @@
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="116" spans="2:6">
+    <row r="24" customFormat="1" ht="120" spans="2:6">
       <c r="B24" s="4" t="s">
         <v>88</v>
       </c>
@@ -9239,7 +9312,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="72.5" spans="2:6">
+    <row r="25" customFormat="1" ht="75" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
@@ -9252,7 +9325,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="29" spans="2:6">
+    <row r="26" customFormat="1" ht="30" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>90</v>
       </c>
@@ -9263,7 +9336,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="29" spans="2:6">
+    <row r="27" customFormat="1" ht="30" spans="2:6">
       <c r="B27" s="4" t="s">
         <v>92</v>
       </c>
@@ -9274,7 +9347,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="29" spans="2:6">
+    <row r="28" customFormat="1" ht="30" spans="2:6">
       <c r="B28" s="4" t="s">
         <v>94</v>
       </c>
@@ -9285,7 +9358,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="29" spans="2:6">
+    <row r="29" customFormat="1" ht="30" spans="2:6">
       <c r="B29" s="4" t="s">
         <v>96</v>
       </c>
@@ -9296,7 +9369,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="29" spans="2:6">
+    <row r="30" customFormat="1" ht="30" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>98</v>
       </c>
@@ -9345,13 +9418,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
-    <col min="3" max="3" width="46.8545454545455" customWidth="1"/>
-    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
-    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
+    <col min="3" max="3" width="46.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
+    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9375,7 +9448,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="43.5" spans="1:1">
+    <row r="2" ht="45" spans="1:1">
       <c r="A2" s="21" t="s">
         <v>348</v>
       </c>
@@ -9413,7 +9486,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="29" spans="2:6">
+    <row r="6" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9435,7 +9508,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="145" spans="2:5">
+    <row r="8" ht="150" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9460,7 +9533,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="10" ht="29" spans="2:4">
+    <row r="10" ht="30" spans="2:4">
       <c r="B10" s="5" t="s">
         <v>359</v>
       </c>
@@ -9479,7 +9552,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="29" spans="2:4">
+    <row r="12" ht="30" spans="2:4">
       <c r="B12" s="5" t="s">
         <v>362</v>
       </c>
@@ -9499,7 +9572,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="14" ht="29" spans="2:4">
+    <row r="14" ht="30" spans="2:4">
       <c r="B14" s="4" t="s">
         <v>366</v>
       </c>
@@ -9520,7 +9593,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="16" ht="58" spans="2:4">
+    <row r="16" ht="75" spans="2:4">
       <c r="B16" s="5" t="s">
         <v>269</v>
       </c>
@@ -9531,7 +9604,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" ht="29" spans="2:3">
+    <row r="17" ht="30" spans="2:3">
       <c r="B17" s="5" t="s">
         <v>271</v>
       </c>
@@ -9539,7 +9612,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="18" ht="87" spans="2:5">
+    <row r="18" ht="90" spans="2:5">
       <c r="B18" t="s">
         <v>371</v>
       </c>
@@ -9599,14 +9672,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9650,7 +9723,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="4" ht="82.5" spans="1:5">
+    <row r="4" ht="78" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -9675,7 +9748,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -9697,7 +9770,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="101.5" spans="2:5">
+    <row r="8" ht="105" spans="2:5">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -9722,7 +9795,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="10" ht="43.5" spans="2:5">
+    <row r="10" ht="45" spans="2:5">
       <c r="B10" s="5" t="s">
         <v>219</v>
       </c>
@@ -9734,7 +9807,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="11" ht="203" spans="2:5">
+    <row r="11" ht="210" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -9743,7 +9816,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="12" ht="203" spans="2:5">
+    <row r="12" ht="210" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
@@ -9795,7 +9868,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="29" spans="2:5">
+    <row r="17" ht="30" spans="2:5">
       <c r="B17" s="5" t="s">
         <v>362</v>
       </c>
@@ -9807,7 +9880,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="18" ht="101.5" spans="2:5">
+    <row r="18" ht="105" spans="2:5">
       <c r="B18" s="4" t="s">
         <v>363</v>
       </c>
@@ -9821,7 +9894,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="19" ht="29" spans="2:3">
+    <row r="19" ht="30" spans="2:3">
       <c r="B19" s="4" t="s">
         <v>366</v>
       </c>
@@ -9829,7 +9902,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="20" ht="29" spans="2:3">
+    <row r="20" ht="30" spans="2:3">
       <c r="B20" s="4" t="s">
         <v>368</v>
       </c>
@@ -9849,7 +9922,7 @@
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="72.5" spans="2:5">
+    <row r="22" ht="75" spans="2:5">
       <c r="B22" s="5" t="s">
         <v>406</v>
       </c>
@@ -9861,7 +9934,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="23" ht="43.5" spans="2:5">
+    <row r="23" ht="45" spans="2:5">
       <c r="B23" s="5" t="s">
         <v>409</v>
       </c>
@@ -9870,7 +9943,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="24" ht="58" spans="2:4">
+    <row r="24" ht="75" spans="2:4">
       <c r="B24" s="5" t="s">
         <v>269</v>
       </c>
@@ -9881,7 +9954,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" ht="29" spans="2:3">
+    <row r="25" ht="30" spans="2:3">
       <c r="B25" s="5" t="s">
         <v>271</v>
       </c>
@@ -9889,7 +9962,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="26" ht="43.5" spans="2:4">
+    <row r="26" ht="45" spans="2:4">
       <c r="B26" s="5" t="s">
         <v>411</v>
       </c>
@@ -9900,7 +9973,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="27" ht="203" spans="2:5">
+    <row r="27" ht="210" spans="2:5">
       <c r="B27" s="5" t="s">
         <v>371</v>
       </c>
@@ -9912,7 +9985,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="28" ht="43.5" spans="2:4">
+    <row r="28" ht="45" spans="2:4">
       <c r="B28" s="5" t="s">
         <v>415</v>
       </c>
@@ -9972,14 +10045,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
-    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -10047,7 +10120,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="29" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -10072,7 +10145,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" ht="101.5" spans="2:6">
+    <row r="8" ht="105" spans="2:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
@@ -10098,7 +10171,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="10" ht="159.5" spans="2:5">
+    <row r="10" ht="165" spans="2:5">
       <c r="B10" s="5" t="s">
         <v>356</v>
       </c>
@@ -10112,7 +10185,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="11" ht="159.5" spans="2:5">
+    <row r="11" ht="180" spans="2:5">
       <c r="B11" s="5" t="s">
         <v>359</v>
       </c>
@@ -10121,7 +10194,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="12" ht="145" spans="2:5">
+    <row r="12" ht="150" spans="2:5">
       <c r="B12" s="5" t="s">
         <v>361</v>
       </c>
@@ -10130,7 +10203,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="13" ht="58" spans="2:4">
+    <row r="13" ht="75" spans="2:4">
       <c r="B13" s="5" t="s">
         <v>269</v>
       </c>
@@ -10141,7 +10214,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" ht="29" spans="2:3">
+    <row r="14" ht="30" spans="2:3">
       <c r="B14" s="5" t="s">
         <v>271</v>
       </c>
@@ -10149,7 +10222,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" ht="43.5" spans="2:4">
+    <row r="15" ht="45" spans="2:4">
       <c r="B15" s="5" t="s">
         <v>411</v>
       </c>
@@ -10160,7 +10233,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="16" ht="203" spans="2:5">
+    <row r="16" ht="210" spans="2:5">
       <c r="B16" s="5" t="s">
         <v>371</v>
       </c>
@@ -10172,7 +10245,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="17" ht="43.5" spans="2:4">
+    <row r="17" ht="45" spans="2:4">
       <c r="B17" s="5" t="s">
         <v>415</v>
       </c>
@@ -10197,7 +10270,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="19" ht="159.5" spans="2:5">
+    <row r="19" ht="165" spans="2:5">
       <c r="B19" t="s">
         <v>428</v>
       </c>

</xml_diff>

<commit_message>
feat: move XSLT and channel files updates for CCDA and HL7 to integration artifacts and update specification documents #2909
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="450">
   <si>
     <t>AthenaHealth CCDA</t>
   </si>
@@ -689,6 +689,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">If </t>
     </r>
     <r>
@@ -3659,13 +3666,10 @@
     <t>name</t>
   </si>
   <si>
-    <t>ClinicalDocument.component.structuredBody.component.section[@ID='encounters'].entry[1].encounter.participant[@typeCode='LOC'].participantRole[@classCode='SDLOC'].playingEntity.name</t>
+    <t>Document.author.assignedAuthor.representedOrganization.name</t>
   </si>
   <si>
     <t>"name" : "Care Ridge SCN",</t>
-  </si>
-  <si>
-    <t>If the name is not available in the provided xpath, then it will take from `Document.author.assignedAuthor.representedOrganization.name`.</t>
   </si>
   <si>
     <t>type -&gt; code</t>
@@ -6018,6 +6022,7 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6026,6 +6031,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6057,17 +6070,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6657,7 +6661,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -7185,7 +7189,7 @@
     <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="1:3">
       <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
@@ -7265,7 +7269,7 @@
     <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:6">
+    <row r="1" s="1" customFormat="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -7285,26 +7289,26 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="29" customHeight="1" spans="1:5">
+    <row r="2" ht="29" customHeight="1" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="2:3">
+    <row r="3" spans="1:7">
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="4" ht="60" spans="2:7">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="4" ht="60" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7312,12 +7316,12 @@
         <v>17</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="1:7">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
@@ -7326,118 +7330,118 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="30" spans="1:7">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>434</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6">
+    </row>
+    <row r="7" spans="1:7">
       <c r="B7" s="5" t="s">
         <v>324</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="D7" t="s">
         <v>437</v>
-      </c>
-      <c r="D7" t="s">
-        <v>438</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="1" ht="75" spans="2:5">
+    <row r="8" customFormat="1" ht="75" spans="1:7">
       <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>86</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" ht="60" spans="2:5">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="60" spans="1:7">
       <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" customFormat="1" spans="2:5">
+    <row r="10" customFormat="1" spans="1:7">
       <c r="B10" s="4" t="s">
         <v>90</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="4"/>
     </row>
-    <row r="11" customFormat="1" spans="2:5">
+    <row r="11" customFormat="1" spans="1:7">
       <c r="B11" s="4" t="s">
         <v>92</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="4"/>
     </row>
-    <row r="12" customFormat="1" spans="2:5">
+    <row r="12" customFormat="1" spans="1:7">
       <c r="B12" s="4" t="s">
         <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="4"/>
     </row>
-    <row r="13" customFormat="1" spans="2:5">
+    <row r="13" customFormat="1" spans="1:7">
       <c r="B13" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" customFormat="1" spans="2:5">
+    <row r="14" customFormat="1" spans="1:7">
       <c r="B14" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" customFormat="1" spans="2:5">
+    <row r="15" customFormat="1" spans="1:7">
       <c r="B15" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>447</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>448</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" customFormat="1" spans="2:6">
+    <row r="16" customFormat="1" spans="1:7">
       <c r="B16" s="4" t="s">
         <v>192</v>
       </c>
@@ -7445,7 +7449,7 @@
         <v>193</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="4"/>
@@ -7455,7 +7459,7 @@
         <v>195</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="8"/>
@@ -7506,12 +7510,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="1:3">
+    <row r="3" customFormat="1" spans="1:6">
       <c r="A3" s="1"/>
       <c r="B3" t="s">
         <v>14</v>
@@ -7520,7 +7524,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="1" spans="1:4">
+    <row r="4" customFormat="1" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
         <v>16</v>
@@ -7532,7 +7536,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" s="27" customFormat="1" ht="61" customHeight="1" spans="1:4">
+    <row r="5" s="27" customFormat="1" ht="61" customHeight="1" spans="1:6">
       <c r="A5" s="28"/>
       <c r="B5" s="28" t="s">
         <v>19</v>
@@ -7544,7 +7548,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" s="27" customFormat="1" ht="49" customHeight="1" spans="1:4">
+    <row r="6" s="27" customFormat="1" ht="49" customHeight="1" spans="1:6">
       <c r="A6" s="28"/>
       <c r="B6" s="28" t="s">
         <v>22</v>
@@ -7554,7 +7558,7 @@
       </c>
       <c r="D6" s="29"/>
     </row>
-    <row r="7" s="27" customFormat="1" ht="86" customHeight="1" spans="1:4">
+    <row r="7" s="27" customFormat="1" ht="86" customHeight="1" spans="1:6">
       <c r="A7" s="28"/>
       <c r="B7" s="28" t="s">
         <v>24</v>
@@ -7564,7 +7568,7 @@
       </c>
       <c r="D7" s="29"/>
     </row>
-    <row r="8" customFormat="1" spans="2:4">
+    <row r="8" customFormat="1" spans="1:6">
       <c r="B8" t="s">
         <v>26</v>
       </c>
@@ -7573,7 +7577,7 @@
       </c>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" customFormat="1" spans="2:3">
+    <row r="9" customFormat="1" spans="1:6">
       <c r="B9" t="s">
         <v>28</v>
       </c>
@@ -7581,7 +7585,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" customFormat="1" ht="30" spans="2:3">
+    <row r="10" customFormat="1" ht="30" spans="1:6">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7589,12 +7593,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:1">
+    <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="2:3">
+    <row r="15" spans="1:6">
       <c r="B15" t="s">
         <v>33</v>
       </c>
@@ -7602,7 +7606,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="2:3">
+    <row r="16" ht="75" spans="1:6">
       <c r="B16" t="s">
         <v>35</v>
       </c>
@@ -7610,7 +7614,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="2:3">
+    <row r="17" spans="2:5">
       <c r="B17" t="s">
         <v>37</v>
       </c>
@@ -7653,7 +7657,7 @@
       </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" ht="105" spans="2:3">
+    <row r="22" ht="105" spans="2:5">
       <c r="B22" s="31" t="s">
         <v>47</v>
       </c>
@@ -7707,12 +7711,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:6">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>14</v>
@@ -7721,7 +7725,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="2:4">
+    <row r="4" spans="1:6">
       <c r="B4" s="15" t="s">
         <v>16</v>
       </c>
@@ -7732,7 +7736,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:6">
       <c r="A5" s="1"/>
       <c r="B5" s="15" t="s">
         <v>19</v>
@@ -7741,7 +7745,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:3">
+    <row r="6" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -7749,7 +7753,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" ht="30" spans="2:4">
+    <row r="7" ht="30" spans="1:6">
       <c r="B7" s="4" t="s">
         <v>55</v>
       </c>
@@ -7760,7 +7764,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" ht="60" spans="2:5">
+    <row r="8" ht="60" spans="1:6">
       <c r="B8" s="4" t="s">
         <v>58</v>
       </c>
@@ -7774,7 +7778,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
+    <row r="9" spans="1:6">
       <c r="B9" s="10" t="s">
         <v>62</v>
       </c>
@@ -7783,7 +7787,7 @@
       </c>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="2:4">
+    <row r="10" spans="1:6">
       <c r="B10" s="4" t="s">
         <v>64</v>
       </c>
@@ -7794,7 +7798,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="2:4">
+    <row r="11" spans="1:6">
       <c r="B11" s="15" t="s">
         <v>67</v>
       </c>
@@ -7805,7 +7809,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="2:4">
+    <row r="12" spans="1:6">
       <c r="B12" s="15" t="s">
         <v>70</v>
       </c>
@@ -7816,7 +7820,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" ht="60" spans="2:4">
+    <row r="13" ht="60" spans="1:6">
       <c r="B13" s="4" t="s">
         <v>72</v>
       </c>
@@ -7827,7 +7831,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="2:4">
+    <row r="14" ht="30" spans="1:6">
       <c r="B14" s="4" t="s">
         <v>75</v>
       </c>
@@ -7838,7 +7842,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" ht="30" spans="2:4">
+    <row r="15" ht="30" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>78</v>
       </c>
@@ -7849,7 +7853,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="2:4">
+    <row r="16" spans="1:6">
       <c r="B16" s="15" t="s">
         <v>81</v>
       </c>
@@ -7874,7 +7878,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="18" ht="60" spans="2:4">
+    <row r="18" ht="60" spans="2:5">
       <c r="B18" s="4" t="s">
         <v>88</v>
       </c>
@@ -7883,7 +7887,7 @@
       </c>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="2:4">
+    <row r="19" spans="2:5">
       <c r="B19" s="4" t="s">
         <v>90</v>
       </c>
@@ -7892,7 +7896,7 @@
       </c>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="2:4">
+    <row r="20" spans="2:5">
       <c r="B20" s="4" t="s">
         <v>92</v>
       </c>
@@ -7901,7 +7905,7 @@
       </c>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="2:4">
+    <row r="21" spans="2:5">
       <c r="B21" s="4" t="s">
         <v>94</v>
       </c>
@@ -7910,7 +7914,7 @@
       </c>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="2:4">
+    <row r="22" spans="2:5">
       <c r="B22" s="4" t="s">
         <v>96</v>
       </c>
@@ -7919,7 +7923,7 @@
       </c>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="2:4">
+    <row r="23" spans="2:5">
       <c r="B23" s="4" t="s">
         <v>98</v>
       </c>
@@ -7939,7 +7943,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" spans="2:3">
+    <row r="25" spans="2:5">
       <c r="B25" s="4" t="s">
         <v>103</v>
       </c>
@@ -8026,7 +8030,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" ht="30" spans="2:4">
+    <row r="33" ht="30" spans="2:6">
       <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
@@ -8035,7 +8039,7 @@
       </c>
       <c r="D33" s="14"/>
     </row>
-    <row r="34" spans="2:4">
+    <row r="34" spans="2:6">
       <c r="B34" s="4" t="s">
         <v>114</v>
       </c>
@@ -8044,7 +8048,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" ht="30" spans="2:4">
+    <row r="35" ht="30" spans="2:6">
       <c r="B35" s="4" t="s">
         <v>116</v>
       </c>
@@ -8053,7 +8057,7 @@
       </c>
       <c r="D35" s="14"/>
     </row>
-    <row r="36" spans="2:4">
+    <row r="36" spans="2:6">
       <c r="B36" s="4" t="s">
         <v>118</v>
       </c>
@@ -8062,7 +8066,7 @@
       </c>
       <c r="D36" s="14"/>
     </row>
-    <row r="37" spans="2:4">
+    <row r="37" spans="2:6">
       <c r="B37" s="4" t="s">
         <v>118</v>
       </c>
@@ -8073,7 +8077,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" ht="45" spans="2:5">
+    <row r="38" ht="45" spans="2:6">
       <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
@@ -8107,7 +8111,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="2:4">
+    <row r="41" spans="2:6">
       <c r="B41" s="15" t="s">
         <v>136</v>
       </c>
@@ -8116,7 +8120,7 @@
       </c>
       <c r="D41" s="10"/>
     </row>
-    <row r="42" spans="2:4">
+    <row r="42" spans="2:6">
       <c r="B42" s="15" t="s">
         <v>138</v>
       </c>
@@ -8125,7 +8129,7 @@
       </c>
       <c r="D42" s="10"/>
     </row>
-    <row r="43" spans="2:4">
+    <row r="43" spans="2:6">
       <c r="B43" s="15" t="s">
         <v>140</v>
       </c>
@@ -8134,7 +8138,7 @@
       </c>
       <c r="D43" s="10"/>
     </row>
-    <row r="44" spans="2:4">
+    <row r="44" spans="2:6">
       <c r="B44" s="4" t="s">
         <v>142</v>
       </c>
@@ -8143,7 +8147,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="195" spans="2:5">
+    <row r="45" ht="195" spans="2:6">
       <c r="B45" s="15" t="s">
         <v>143</v>
       </c>
@@ -8157,7 +8161,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="46" ht="195" spans="2:5">
+    <row r="46" ht="195" spans="2:6">
       <c r="B46" s="15" t="s">
         <v>147</v>
       </c>
@@ -8171,7 +8175,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" ht="195" spans="2:5">
+    <row r="47" ht="195" spans="2:6">
       <c r="B47" s="15" t="s">
         <v>151</v>
       </c>
@@ -8183,7 +8187,7 @@
       </c>
       <c r="E47" s="25"/>
     </row>
-    <row r="48" customFormat="1" spans="2:5">
+    <row r="48" customFormat="1" spans="2:6">
       <c r="B48" s="4" t="s">
         <v>154</v>
       </c>
@@ -8193,7 +8197,7 @@
       <c r="D48" s="10"/>
       <c r="E48" s="4"/>
     </row>
-    <row r="49" customFormat="1" spans="2:5">
+    <row r="49" customFormat="1" spans="2:6">
       <c r="B49" s="4" t="s">
         <v>155</v>
       </c>
@@ -8203,7 +8207,7 @@
       <c r="D49" s="10"/>
       <c r="E49" s="4"/>
     </row>
-    <row r="50" customFormat="1" spans="2:5">
+    <row r="50" customFormat="1" spans="2:6">
       <c r="B50" s="4" t="s">
         <v>157</v>
       </c>
@@ -8213,7 +8217,7 @@
       <c r="D50" s="10"/>
       <c r="E50" s="4"/>
     </row>
-    <row r="51" customFormat="1" spans="2:5">
+    <row r="51" customFormat="1" spans="2:6">
       <c r="B51" s="4" t="s">
         <v>159</v>
       </c>
@@ -8223,7 +8227,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="150" spans="2:5">
+    <row r="52" ht="150" spans="2:6">
       <c r="B52" s="10" t="s">
         <v>160</v>
       </c>
@@ -8237,7 +8241,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="2:5">
+    <row r="53" spans="2:6">
       <c r="B53" s="4" t="s">
         <v>164</v>
       </c>
@@ -8247,7 +8251,7 @@
       <c r="D53" s="10"/>
       <c r="E53" s="8"/>
     </row>
-    <row r="54" customFormat="1" spans="2:5">
+    <row r="54" customFormat="1" spans="2:6">
       <c r="B54" s="4" t="s">
         <v>166</v>
       </c>
@@ -8257,7 +8261,7 @@
       <c r="D54" s="10"/>
       <c r="E54" s="8"/>
     </row>
-    <row r="55" customFormat="1" spans="2:5">
+    <row r="55" customFormat="1" spans="2:6">
       <c r="B55" s="4" t="s">
         <v>167</v>
       </c>
@@ -8267,7 +8271,7 @@
       <c r="D55" s="10"/>
       <c r="E55" s="8"/>
     </row>
-    <row r="56" customFormat="1" spans="2:5">
+    <row r="56" customFormat="1" spans="2:6">
       <c r="B56" s="4" t="s">
         <v>169</v>
       </c>
@@ -8277,7 +8281,7 @@
       <c r="D56" s="10"/>
       <c r="E56" s="8"/>
     </row>
-    <row r="57" customFormat="1" spans="2:5">
+    <row r="57" customFormat="1" spans="2:6">
       <c r="B57" s="4" t="s">
         <v>171</v>
       </c>
@@ -8287,7 +8291,7 @@
       <c r="D57" s="10"/>
       <c r="E57" s="8"/>
     </row>
-    <row r="58" spans="2:5">
+    <row r="58" spans="2:6">
       <c r="B58" s="4" t="s">
         <v>172</v>
       </c>
@@ -8297,7 +8301,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="8"/>
     </row>
-    <row r="59" ht="180" spans="2:5">
+    <row r="59" ht="180" spans="2:6">
       <c r="B59" s="10" t="s">
         <v>174</v>
       </c>
@@ -8430,7 +8434,7 @@
     <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:6">
+    <row r="1" s="1" customFormat="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -8450,7 +8454,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="105" customHeight="1" spans="1:5">
+    <row r="2" ht="105" customHeight="1" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
@@ -8461,7 +8465,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="2:3">
+    <row r="3" spans="1:7">
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
@@ -8469,7 +8473,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" ht="60" spans="2:7">
+    <row r="4" ht="60" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8482,7 +8486,7 @@
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="1:7">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
@@ -8491,7 +8495,7 @@
       </c>
       <c r="E5" s="8"/>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="1:7">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -8500,7 +8504,7 @@
       </c>
       <c r="E6" s="26"/>
     </row>
-    <row r="7" ht="120" spans="2:6">
+    <row r="7" ht="120" spans="1:7">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8515,7 +8519,7 @@
       </c>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" ht="94" customHeight="1" spans="2:5">
+    <row r="8" ht="94" customHeight="1" spans="1:7">
       <c r="B8" s="5" t="s">
         <v>206</v>
       </c>
@@ -8529,7 +8533,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="9" customFormat="1" spans="2:5">
+    <row r="9" customFormat="1" spans="1:7">
       <c r="B9" s="5" t="s">
         <v>210</v>
       </c>
@@ -8541,7 +8545,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="1:7">
       <c r="B10" s="5" t="s">
         <v>212</v>
       </c>
@@ -8553,7 +8557,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="11" ht="225" spans="2:5">
+    <row r="11" ht="225" spans="1:7">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
@@ -8567,7 +8571,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" spans="1:7">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
@@ -8578,7 +8582,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="13" spans="2:5">
+    <row r="13" spans="1:7">
       <c r="B13" s="5" t="s">
         <v>219</v>
       </c>
@@ -8589,7 +8593,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="14" ht="45" spans="2:5">
+    <row r="14" ht="45" spans="1:7">
       <c r="B14" s="5" t="s">
         <v>221</v>
       </c>
@@ -8603,7 +8607,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" ht="255" spans="2:5">
+    <row r="15" ht="255" spans="1:7">
       <c r="B15" s="5" t="s">
         <v>225</v>
       </c>
@@ -8617,7 +8621,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="16" ht="45" spans="2:5">
+    <row r="16" ht="45" spans="1:7">
       <c r="B16" s="5" t="s">
         <v>229</v>
       </c>
@@ -8629,7 +8633,7 @@
       </c>
       <c r="E16" s="8"/>
     </row>
-    <row r="17" ht="45" spans="2:5">
+    <row r="17" ht="45" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>232</v>
       </c>
@@ -8641,7 +8645,7 @@
       </c>
       <c r="E17" s="8"/>
     </row>
-    <row r="18" ht="45" spans="2:5">
+    <row r="18" ht="45" spans="2:6">
       <c r="B18" t="s">
         <v>235</v>
       </c>
@@ -8655,7 +8659,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="19" ht="60" spans="2:5">
+    <row r="19" ht="60" spans="2:6">
       <c r="B19" s="5" t="s">
         <v>238</v>
       </c>
@@ -8669,7 +8673,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="20" customFormat="1" spans="2:5">
+    <row r="20" customFormat="1" spans="2:6">
       <c r="B20" s="5" t="s">
         <v>241</v>
       </c>
@@ -8750,7 +8754,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:5">
+    <row r="2" ht="18" customHeight="1" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>35</v>
       </c>
@@ -8761,7 +8765,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" customFormat="1" spans="2:3">
+    <row r="3" customFormat="1" spans="1:6">
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
@@ -8769,7 +8773,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" ht="75" spans="1:5">
+    <row r="4" ht="75" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8796,7 +8800,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
@@ -8807,7 +8811,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="255" spans="2:5">
+    <row r="7" ht="255" spans="1:6">
       <c r="B7" s="5" t="s">
         <v>202</v>
       </c>
@@ -8821,7 +8825,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="8" ht="71" customHeight="1" spans="2:5">
+    <row r="8" ht="71" customHeight="1" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>253</v>
       </c>
@@ -8833,7 +8837,7 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" ht="30" spans="2:5">
+    <row r="9" ht="30" spans="1:6">
       <c r="B9" s="5" t="s">
         <v>256</v>
       </c>
@@ -8843,7 +8847,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="25"/>
     </row>
-    <row r="10" spans="2:5">
+    <row r="10" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>258</v>
       </c>
@@ -8853,7 +8857,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" ht="30" spans="2:4">
+    <row r="11" ht="30" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>260</v>
       </c>
@@ -8864,7 +8868,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="12" ht="60" spans="2:5">
+    <row r="12" ht="60" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>263</v>
       </c>
@@ -8873,7 +8877,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="13" ht="33" customHeight="1" spans="2:4">
+    <row r="13" ht="33" customHeight="1" spans="1:6">
       <c r="B13" s="5" t="s">
         <v>265</v>
       </c>
@@ -8882,7 +8886,7 @@
       </c>
       <c r="D13" s="12"/>
     </row>
-    <row r="14" customFormat="1" spans="2:3">
+    <row r="14" customFormat="1" spans="1:6">
       <c r="B14" t="s">
         <v>267</v>
       </c>
@@ -8890,7 +8894,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="60" spans="2:4">
+    <row r="15" customFormat="1" ht="60" spans="1:6">
       <c r="B15" s="5" t="s">
         <v>269</v>
       </c>
@@ -8901,7 +8905,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="2:3">
+    <row r="16" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>271</v>
       </c>
@@ -8909,7 +8913,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" ht="60" spans="2:4">
+    <row r="17" ht="60" spans="2:5">
       <c r="B17" t="s">
         <v>273</v>
       </c>
@@ -8920,7 +8924,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="18" spans="2:3">
+    <row r="18" spans="2:5">
       <c r="B18" t="s">
         <v>276</v>
       </c>
@@ -8993,7 +8997,7 @@
       <c r="D24" s="10"/>
       <c r="E24" s="4"/>
     </row>
-    <row r="25" customFormat="1" spans="2:4">
+    <row r="25" customFormat="1" spans="2:5">
       <c r="B25" s="4" t="s">
         <v>192</v>
       </c>
@@ -9004,7 +9008,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="26" customFormat="1" ht="46" customHeight="1" spans="2:4">
+    <row r="26" customFormat="1" ht="46" customHeight="1" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>195</v>
       </c>
@@ -9061,12 +9065,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" customFormat="1" spans="2:3">
+    <row r="3" customFormat="1" spans="1:6">
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
@@ -9074,7 +9078,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
+    <row r="4" spans="1:6">
       <c r="B4" t="s">
         <v>16</v>
       </c>
@@ -9096,7 +9100,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -9107,7 +9111,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="1:6">
       <c r="B7" s="5" t="s">
         <v>299</v>
       </c>
@@ -9121,7 +9125,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="8" ht="63" customHeight="1" spans="2:6">
+    <row r="8" ht="63" customHeight="1" spans="1:6">
       <c r="B8" t="s">
         <v>303</v>
       </c>
@@ -9135,7 +9139,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="9" spans="2:5">
+    <row r="9" spans="1:6">
       <c r="B9" t="s">
         <v>307</v>
       </c>
@@ -9145,7 +9149,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" ht="30" spans="2:5">
+    <row r="10" ht="30" spans="1:6">
       <c r="B10" s="4" t="s">
         <v>309</v>
       </c>
@@ -9155,7 +9159,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" ht="30" spans="2:5">
+    <row r="11" ht="30" spans="1:6">
       <c r="B11" s="4" t="s">
         <v>311</v>
       </c>
@@ -9165,7 +9169,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:5">
+    <row r="12" ht="30" spans="1:6">
       <c r="B12" s="4" t="s">
         <v>312</v>
       </c>
@@ -9175,7 +9179,7 @@
       <c r="D12" s="10"/>
       <c r="E12" s="8"/>
     </row>
-    <row r="13" customFormat="1" ht="66" customHeight="1" spans="2:6">
+    <row r="13" customFormat="1" ht="66" customHeight="1" spans="1:6">
       <c r="B13" t="s">
         <v>314</v>
       </c>
@@ -9189,7 +9193,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="14" customFormat="1" spans="2:5">
+    <row r="14" customFormat="1" spans="1:6">
       <c r="B14" t="s">
         <v>317</v>
       </c>
@@ -9199,7 +9203,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" customFormat="1" ht="30" spans="2:5">
+    <row r="15" customFormat="1" ht="30" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>319</v>
       </c>
@@ -9209,7 +9213,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="22"/>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="2:5">
+    <row r="16" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="4" t="s">
         <v>321</v>
       </c>
@@ -9219,7 +9223,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="30" spans="2:4">
+    <row r="17" customFormat="1" ht="30" spans="2:6">
       <c r="B17" s="4" t="s">
         <v>322</v>
       </c>
@@ -9228,7 +9232,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="60" spans="2:5">
+    <row r="18" ht="30" spans="2:6">
       <c r="B18" s="5" t="s">
         <v>324</v>
       </c>
@@ -9238,29 +9242,27 @@
       <c r="D18" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>327</v>
-      </c>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" ht="93" customHeight="1" spans="2:6">
       <c r="B19" t="s">
+        <v>327</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="F19" s="8" t="s">
         <v>329</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="2:6">
       <c r="B20" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="10"/>
       <c r="F20" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="21" customFormat="1" ht="120" spans="2:6">
@@ -9269,7 +9271,7 @@
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E21" s="18" t="s">
         <v>102</v>
@@ -9281,7 +9283,7 @@
         <v>103</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
@@ -9291,11 +9293,11 @@
         <v>105</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="23" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F23" s="4"/>
     </row>
@@ -9304,10 +9306,10 @@
         <v>88</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>337</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>338</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
@@ -9317,11 +9319,11 @@
         <v>84</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D25" s="10"/>
       <c r="E25" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F25" s="4"/>
     </row>
@@ -9330,7 +9332,7 @@
         <v>90</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="4"/>
@@ -9341,7 +9343,7 @@
         <v>92</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D27" s="10"/>
       <c r="E27" s="4"/>
@@ -9352,7 +9354,7 @@
         <v>94</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="4"/>
@@ -9363,7 +9365,7 @@
         <v>96</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="4"/>
@@ -9374,13 +9376,13 @@
         <v>98</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D30" s="10"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" customFormat="1" spans="2:4">
+    <row r="31" customFormat="1" spans="2:6">
       <c r="B31" s="4" t="s">
         <v>192</v>
       </c>
@@ -9388,15 +9390,15 @@
         <v>193</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="32" customFormat="1" ht="46" customHeight="1" spans="2:4">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="32" customFormat="1" ht="46" customHeight="1" spans="2:6">
       <c r="B32" s="4" t="s">
         <v>195</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D32" s="14"/>
     </row>
@@ -9448,21 +9450,21 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="45" spans="1:1">
+    <row r="2" ht="45" spans="1:6">
       <c r="A2" s="21" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -9471,7 +9473,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -9486,18 +9488,18 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="30" spans="2:6">
+    <row r="6" ht="30" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="1:6">
       <c r="B7" t="s">
         <v>55</v>
       </c>
@@ -9505,46 +9507,46 @@
         <v>57</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="8" ht="150" spans="2:5">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="8" ht="150" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="D8" t="s">
         <v>353</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="11" t="s">
         <v>354</v>
       </c>
-      <c r="E8" s="11" t="s">
+    </row>
+    <row r="9" ht="70" customHeight="1" spans="1:6">
+      <c r="B9" s="5" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="9" ht="70" customHeight="1" spans="2:4">
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>356</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="D9" s="10" t="s">
+    </row>
+    <row r="10" ht="30" spans="1:6">
+      <c r="B10" s="5" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="10" ht="30" spans="2:4">
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="10"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="B11" s="5" t="s">
         <v>360</v>
-      </c>
-      <c r="D10" s="10"/>
-    </row>
-    <row r="11" spans="2:5">
-      <c r="B11" s="5" t="s">
-        <v>361</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>220</v>
@@ -9552,48 +9554,48 @@
       <c r="D11" s="10"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" ht="30" spans="2:4">
+    <row r="12" ht="30" spans="1:6">
       <c r="B12" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" ht="38" customHeight="1" spans="1:6">
+      <c r="B13" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>360</v>
-      </c>
-      <c r="D12" s="10"/>
-    </row>
-    <row r="13" ht="38" customHeight="1" spans="2:4">
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="10" t="s">
         <v>364</v>
       </c>
-      <c r="D13" s="10" t="s">
+    </row>
+    <row r="14" ht="30" spans="1:6">
+      <c r="B14" s="4" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="14" ht="30" spans="2:4">
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" ht="153" customHeight="1" spans="1:6">
+      <c r="B15" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" ht="153" customHeight="1" spans="2:5">
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>368</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>369</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="8" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="16" ht="75" spans="2:4">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="16" ht="75" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>269</v>
       </c>
@@ -9604,7 +9606,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" ht="30" spans="2:3">
+    <row r="17" ht="30" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>271</v>
       </c>
@@ -9612,32 +9614,32 @@
         <v>272</v>
       </c>
     </row>
-    <row r="18" ht="90" spans="2:5">
+    <row r="18" ht="90" spans="2:6">
       <c r="B18" t="s">
+        <v>370</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" t="s">
         <v>372</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" s="4" t="s">
         <v>373</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="19" spans="2:6">
       <c r="B19" t="s">
+        <v>374</v>
+      </c>
+      <c r="D19" t="s">
         <v>375</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" s="19" t="s">
         <v>376</v>
       </c>
-      <c r="F19" s="19" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4">
+    </row>
+    <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
         <v>192</v>
       </c>
@@ -9645,15 +9647,15 @@
         <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1" spans="2:4">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D21" s="14"/>
     </row>
@@ -9707,32 +9709,32 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="20"/>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:6">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="4" ht="78" spans="1:5">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="4" ht="78" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>381</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>382</v>
       </c>
       <c r="E4" s="18"/>
     </row>
@@ -9748,18 +9750,18 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="1:6">
       <c r="B7" t="s">
         <v>55</v>
       </c>
@@ -9767,90 +9769,90 @@
         <v>57</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="8" ht="105" spans="2:5">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="8" ht="105" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D8" t="s">
+        <v>353</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>384</v>
       </c>
-      <c r="D8" t="s">
-        <v>354</v>
-      </c>
-      <c r="E8" s="16" t="s">
+    </row>
+    <row r="9" ht="139" customHeight="1" spans="1:6">
+      <c r="B9" s="5" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="9" ht="139" customHeight="1" spans="2:5">
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="10" ht="45" spans="2:5">
+    </row>
+    <row r="10" ht="45" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="11" ht="210" spans="2:5">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11" ht="210" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>214</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="11" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="12" ht="210" spans="2:5">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="12" ht="210" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>217</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="11" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="B13" s="5" t="s">
         <v>392</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5">
-      <c r="B13" s="5" t="s">
-        <v>393</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="14" ht="84" customHeight="1" spans="1:6">
+      <c r="B14" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="14" ht="84" customHeight="1" spans="2:5">
-      <c r="B14" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="C14" s="18" t="s">
+      <c r="D14" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E14" s="18" t="s">
         <v>395</v>
       </c>
-      <c r="D14" s="10" t="s">
+    </row>
+    <row r="15" spans="1:6">
+      <c r="B15" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5">
-      <c r="B15" s="5" t="s">
-        <v>359</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>259</v>
@@ -9858,9 +9860,9 @@
       <c r="D15" s="10"/>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>220</v>
@@ -9868,82 +9870,82 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="30" spans="2:5">
+    <row r="17" ht="30" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="8" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="18" ht="105" spans="2:6">
+      <c r="B18" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="18" ht="105" spans="2:5">
-      <c r="B18" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="18" t="s">
         <v>400</v>
       </c>
-      <c r="E18" s="18" t="s">
+    </row>
+    <row r="19" ht="30" spans="2:6">
+      <c r="B19" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="19" ht="30" spans="2:3">
-      <c r="B19" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="20" ht="30" spans="2:3">
+    <row r="20" ht="30" spans="2:6">
       <c r="B20" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C20" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="21" ht="37" customHeight="1" spans="2:5">
+    <row r="21" ht="37" customHeight="1" spans="2:6">
       <c r="B21" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>403</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="12" t="s">
         <v>404</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" ht="75" spans="2:6">
+      <c r="B22" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="E21" s="8"/>
-    </row>
-    <row r="22" ht="75" spans="2:5">
-      <c r="B22" s="5" t="s">
+      <c r="C22" t="s">
         <v>406</v>
-      </c>
-      <c r="C22" t="s">
-        <v>407</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="11" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="23" ht="45" spans="2:6">
+      <c r="B23" s="5" t="s">
         <v>408</v>
-      </c>
-    </row>
-    <row r="23" ht="45" spans="2:5">
-      <c r="B23" s="5" t="s">
-        <v>409</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="11" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="24" ht="75" spans="2:4">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="24" ht="75" spans="2:6">
       <c r="B24" s="5" t="s">
         <v>269</v>
       </c>
@@ -9954,7 +9956,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="25" ht="30" spans="2:3">
+    <row r="25" ht="30" spans="2:6">
       <c r="B25" s="5" t="s">
         <v>271</v>
       </c>
@@ -9962,53 +9964,53 @@
         <v>272</v>
       </c>
     </row>
-    <row r="26" ht="45" spans="2:4">
+    <row r="26" ht="45" spans="2:6">
       <c r="B26" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="C26" t="s">
         <v>411</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="27" ht="210" spans="2:5">
+    </row>
+    <row r="27" ht="210" spans="2:6">
       <c r="B27" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E27" s="18" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="28" ht="45" spans="2:6">
+      <c r="B28" s="5" t="s">
         <v>414</v>
-      </c>
-    </row>
-    <row r="28" ht="45" spans="2:4">
-      <c r="B28" s="5" t="s">
-        <v>415</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="29" spans="2:6">
       <c r="B29" t="s">
+        <v>374</v>
+      </c>
+      <c r="D29" t="s">
         <v>375</v>
-      </c>
-      <c r="D29" t="s">
-        <v>376</v>
       </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>192</v>
       </c>
@@ -10016,15 +10018,15 @@
         <v>193</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="31" ht="46" customHeight="1" spans="2:4">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="31" ht="46" customHeight="1" spans="2:6">
       <c r="B31" s="4" t="s">
         <v>195</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D31" s="14"/>
     </row>
@@ -10080,23 +10082,23 @@
         <v>44</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:6">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -10105,7 +10107,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -10120,18 +10122,18 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="2:6">
+    <row r="6" customFormat="1" ht="30" spans="1:6">
       <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="1:6">
       <c r="B7" t="s">
         <v>55</v>
       </c>
@@ -10139,71 +10141,71 @@
         <v>57</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="8" ht="105" spans="2:6">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="8" ht="105" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D8" t="s">
+        <v>353</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>384</v>
       </c>
-      <c r="D8" t="s">
-        <v>354</v>
-      </c>
-      <c r="E8" s="16" t="s">
+      <c r="F8" s="17"/>
+    </row>
+    <row r="9" ht="409" customHeight="1" spans="1:6">
+      <c r="B9" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="F8" s="17"/>
-    </row>
-    <row r="9" ht="409" customHeight="1" spans="2:5">
-      <c r="B9" s="5" t="s">
-        <v>386</v>
-      </c>
       <c r="D9" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="10" ht="165" spans="2:5">
+    </row>
+    <row r="10" ht="165" spans="1:6">
       <c r="B10" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>254</v>
       </c>
       <c r="D10" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="E10" s="18" t="s">
         <v>423</v>
       </c>
-      <c r="E10" s="18" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="11" ht="180" spans="2:5">
+    </row>
+    <row r="11" ht="180" spans="1:6">
       <c r="B11" s="5" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C11" s="4"/>
       <c r="E11" s="11" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="12" ht="150" spans="2:5">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="12" ht="150" spans="1:6">
       <c r="B12" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C12" s="4"/>
       <c r="E12" s="11" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="13" ht="75" spans="2:4">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" ht="75" spans="1:6">
       <c r="B13" s="5" t="s">
         <v>269</v>
       </c>
@@ -10214,7 +10216,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="2:3">
+    <row r="14" ht="30" spans="1:6">
       <c r="B14" s="5" t="s">
         <v>271</v>
       </c>
@@ -10222,66 +10224,66 @@
         <v>272</v>
       </c>
     </row>
-    <row r="15" ht="45" spans="2:4">
+    <row r="15" ht="45" spans="1:6">
       <c r="B15" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="C15" t="s">
         <v>411</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="16" ht="210" spans="2:5">
+    </row>
+    <row r="16" ht="210" spans="1:6">
       <c r="B16" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E16" s="18" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="17" ht="45" spans="2:6">
+      <c r="B17" s="5" t="s">
         <v>414</v>
-      </c>
-    </row>
-    <row r="17" ht="45" spans="2:4">
-      <c r="B17" s="5" t="s">
-        <v>415</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="18" spans="2:6">
       <c r="B18" t="s">
+        <v>374</v>
+      </c>
+      <c r="D18" t="s">
         <v>375</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>376</v>
       </c>
-      <c r="E18" s="8" t="s">
+    </row>
+    <row r="19" ht="165" spans="2:6">
+      <c r="B19" t="s">
         <v>427</v>
       </c>
-      <c r="F18" s="19" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="19" ht="165" spans="2:5">
-      <c r="B19" t="s">
+      <c r="D19" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" t="s">
         <v>429</v>
       </c>
-      <c r="E19" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4">
+    </row>
+    <row r="20" spans="2:6">
       <c r="B20" s="4" t="s">
         <v>192</v>
       </c>
@@ -10289,15 +10291,15 @@
         <v>193</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="21" ht="46" customHeight="1" spans="2:4">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="21" ht="46" customHeight="1" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>195</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D21" s="14"/>
     </row>

</xml_diff>

<commit_message>
fix: resolve the issue with unknown in Patient Resource marital status which is not displaying in CCDA and HL7 files - Updated the "system" for maritalStatus when the code is "UNK". - Updated the XSLT files for Epic, Medent, AthenaHealth, Generic CCDA and HL7 files. - Updated all the CCDA and HL7 conversion specification documents with the changes.
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -90,6 +90,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Randomly generated UUID which is used as the</t>
     </r>
     <r>
@@ -1784,7 +1791,7 @@
     <t>maritalStatus -&gt; coding -&gt; system</t>
   </si>
   <si>
-    <t>"http://terminology.hl7.org/CodeSystem/v3-MaritalStatus"</t>
+    <t>If maritalStatus code is "UNK" then "http://terminology.hl7.org/CodeSystem/v3-NullFlavor", otherwise "http://terminology.hl7.org/CodeSystem/v3-MaritalStatus".</t>
   </si>
   <si>
     <t>maritalStatus -&gt; coding -&gt; code</t>
@@ -5998,6 +6005,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF00B050"/>
@@ -6009,13 +6023,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6491,7 +6498,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6547,9 +6554,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -7139,18 +7143,18 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="34"/>
+    <col min="1" max="1" width="8.88571428571429" style="33"/>
     <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
     <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="34" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="34">
+      <c r="A3" s="33">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -7161,7 +7165,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="34">
+      <c r="A4" s="33">
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
@@ -7172,10 +7176,10 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="34">
+      <c r="A5" s="33">
         <v>3</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -7183,10 +7187,10 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="34">
+      <c r="A6" s="33">
         <v>4</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="26" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -7194,10 +7198,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="34">
+      <c r="A7" s="33">
         <v>5</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -7485,44 +7489,44 @@
       <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="28" t="s">
         <v>17</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" s="28" customFormat="1" ht="61" customHeight="1" spans="1:6">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30" t="s">
+    <row r="5" s="27" customFormat="1" ht="61" customHeight="1" spans="1:6">
+      <c r="A5" s="29"/>
+      <c r="B5" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" s="28" customFormat="1" ht="49" customHeight="1" spans="1:6">
-      <c r="A6" s="30"/>
-      <c r="B6" s="30" t="s">
+    <row r="6" s="27" customFormat="1" ht="49" customHeight="1" spans="1:6">
+      <c r="A6" s="29"/>
+      <c r="B6" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="31"/>
-    </row>
-    <row r="7" s="28" customFormat="1" ht="316" customHeight="1" spans="1:6">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30" t="s">
+      <c r="D6" s="30"/>
+    </row>
+    <row r="7" s="27" customFormat="1" ht="316" customHeight="1" spans="1:6">
+      <c r="A7" s="29"/>
+      <c r="B7" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="31"/>
+      <c r="D7" s="30"/>
     </row>
     <row r="8" customFormat="1" spans="1:6">
       <c r="B8" t="s">
@@ -7585,7 +7589,7 @@
       <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="6" t="s">
         <v>41</v>
       </c>
     </row>
@@ -7614,7 +7618,7 @@
       <c r="E21" s="9"/>
     </row>
     <row r="22" ht="105" spans="2:5">
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="32" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="11" t="s">
@@ -7651,19 +7655,19 @@
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>50</v>
       </c>
     </row>
@@ -7685,7 +7689,7 @@
       <c r="B4" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -7895,7 +7899,7 @@
       <c r="D24" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="6" t="s">
         <v>103</v>
       </c>
     </row>
@@ -7914,7 +7918,7 @@
       <c r="C26" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="23" t="s">
         <v>108</v>
       </c>
     </row>
@@ -8041,7 +8045,7 @@
         <v>80</v>
       </c>
       <c r="D38" s="15"/>
-      <c r="E38" s="36" t="s">
+      <c r="E38" s="35" t="s">
         <v>130</v>
       </c>
     </row>
@@ -8113,7 +8117,7 @@
       <c r="D45" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="E45" s="19" t="s">
+      <c r="E45" s="6" t="s">
         <v>147</v>
       </c>
     </row>
@@ -8121,7 +8125,7 @@
       <c r="B46" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" s="6" t="s">
         <v>149</v>
       </c>
       <c r="D46" s="11" t="s">
@@ -8141,7 +8145,7 @@
       <c r="D47" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="E47" s="26"/>
+      <c r="E47" s="25"/>
     </row>
     <row r="48" customFormat="1" spans="2:6">
       <c r="B48" s="4" t="s">
@@ -8187,7 +8191,7 @@
       <c r="B52" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="6" t="s">
         <v>162</v>
       </c>
       <c r="D52" s="11" t="s">
@@ -8267,7 +8271,7 @@
       <c r="D59" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="6" t="s">
         <v>177</v>
       </c>
     </row>
@@ -8282,7 +8286,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="61" spans="2:6">
+    <row r="61" ht="45" spans="2:6">
       <c r="B61" s="4" t="s">
         <v>181</v>
       </c>
@@ -8459,7 +8463,7 @@
       <c r="C6" t="s">
         <v>202</v>
       </c>
-      <c r="E6" s="27"/>
+      <c r="E6" s="26"/>
     </row>
     <row r="7" ht="120" spans="1:7">
       <c r="B7" s="5" t="s">
@@ -8568,13 +8572,13 @@
       <c r="B15" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="6" t="s">
         <v>227</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="6" t="s">
         <v>229</v>
       </c>
     </row>
@@ -8698,7 +8702,7 @@
       <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -8735,7 +8739,7 @@
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="6" t="s">
         <v>248</v>
       </c>
       <c r="D4" t="s">
@@ -8766,11 +8770,11 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="255" spans="1:6">
+    <row r="7" ht="225" spans="1:6">
       <c r="B7" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="6" t="s">
         <v>251</v>
       </c>
       <c r="D7" t="s">
@@ -8792,7 +8796,7 @@
       </c>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" ht="30" spans="1:6">
+    <row r="9" spans="1:6">
       <c r="B9" s="5" t="s">
         <v>257</v>
       </c>
@@ -8800,7 +8804,7 @@
         <v>258</v>
       </c>
       <c r="D9" s="11"/>
-      <c r="E9" s="26"/>
+      <c r="E9" s="25"/>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="5" t="s">
@@ -8812,11 +8816,11 @@
       <c r="D10" s="11"/>
       <c r="E10" s="10"/>
     </row>
-    <row r="11" ht="30" spans="1:6">
+    <row r="11" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="6" t="s">
         <v>262</v>
       </c>
       <c r="D11" s="13" t="s">
@@ -8908,7 +8912,7 @@
       <c r="C20" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="E20" s="20"/>
+      <c r="E20" s="19"/>
     </row>
     <row r="21" ht="409.5" spans="2:5">
       <c r="B21" t="s">
@@ -8928,7 +8932,7 @@
       <c r="C22" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="E22" s="23"/>
+      <c r="E22" s="22"/>
     </row>
     <row r="23" ht="66" customHeight="1" spans="2:5">
       <c r="B23" t="s">
@@ -9087,7 +9091,7 @@
       <c r="B8" t="s">
         <v>306</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="6" t="s">
         <v>307</v>
       </c>
       <c r="D8" s="11" t="s">
@@ -9141,7 +9145,7 @@
       <c r="B13" t="s">
         <v>317</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="6" t="s">
         <v>318</v>
       </c>
       <c r="D13" s="11" t="s">
@@ -9159,7 +9163,7 @@
         <v>321</v>
       </c>
       <c r="D14" s="11"/>
-      <c r="E14" s="23"/>
+      <c r="E14" s="22"/>
     </row>
     <row r="15" customFormat="1" ht="30" spans="1:6">
       <c r="B15" s="4" t="s">
@@ -9169,7 +9173,7 @@
         <v>323</v>
       </c>
       <c r="D15" s="11"/>
-      <c r="E15" s="23"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="4" t="s">
@@ -9194,7 +9198,7 @@
       <c r="B18" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="6" t="s">
         <v>328</v>
       </c>
       <c r="D18" s="11" t="s">
@@ -9231,7 +9235,7 @@
       <c r="D21" s="11" t="s">
         <v>335</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="6" t="s">
         <v>103</v>
       </c>
       <c r="F21" s="4"/>
@@ -9254,7 +9258,7 @@
         <v>337</v>
       </c>
       <c r="D23" s="11"/>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="23" t="s">
         <v>338</v>
       </c>
       <c r="F23" s="4"/>
@@ -9409,7 +9413,7 @@
       </c>
     </row>
     <row r="2" ht="45" spans="1:6">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>350</v>
       </c>
     </row>
@@ -9564,7 +9568,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="17" ht="30" spans="2:6">
+    <row r="17" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>272</v>
       </c>
@@ -9593,7 +9597,7 @@
       <c r="D19" t="s">
         <v>379</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="19" t="s">
         <v>380</v>
       </c>
     </row>
@@ -9672,7 +9676,7 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="21"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1"/>
@@ -9688,13 +9692,13 @@
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="6" t="s">
         <v>384</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="E4" s="19"/>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" customFormat="1" spans="1:6">
       <c r="A5" s="1"/>
@@ -9751,7 +9755,7 @@
       <c r="D9" s="7" t="s">
         <v>390</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="6" t="s">
         <v>391</v>
       </c>
     </row>
@@ -9798,13 +9802,13 @@
       <c r="B14" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="6" t="s">
         <v>398</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>361</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="6" t="s">
         <v>399</v>
       </c>
     </row>
@@ -9850,7 +9854,7 @@
       <c r="D18" s="11" t="s">
         <v>403</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="6" t="s">
         <v>404</v>
       </c>
     </row>
@@ -9903,7 +9907,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="24" ht="75" spans="2:6">
+    <row r="24" ht="60" spans="2:6">
       <c r="B24" s="5" t="s">
         <v>270</v>
       </c>
@@ -9941,7 +9945,7 @@
       <c r="D27" t="s">
         <v>376</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="6" t="s">
         <v>417</v>
       </c>
     </row>
@@ -10141,7 +10145,7 @@
       <c r="D10" s="11" t="s">
         <v>427</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="6" t="s">
         <v>428</v>
       </c>
     </row>
@@ -10174,7 +10178,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" spans="1:6">
       <c r="B14" s="5" t="s">
         <v>272</v>
       </c>
@@ -10201,7 +10205,7 @@
       <c r="D16" t="s">
         <v>376</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="6" t="s">
         <v>417</v>
       </c>
     </row>
@@ -10226,7 +10230,7 @@
       <c r="E18" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="19" t="s">
         <v>380</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update CCDA to FHIR convertion specification documents to incorporate the changes #3155
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - AthenaHealth.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="8"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="AthenaHealth" sheetId="11" r:id="rId1"/>
@@ -1914,13 +1914,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -1942,53 +1935,112 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> CCDS, if there is an entry in the Social history section['</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>29762-2'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>] with a consent question (`entry.observation.entryRelationship.observation with code = "105511-0"`) and answer (`entry.observation.entryRelationship.observation.value.code`), then if the `entry.observation.entryRelationship.observation.value.code = '</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>LA33-6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>' then, a consent resource with provision.type = "permit" will be generated. Otherwise, a consent resource with provision.type = "deny" will be generated.
-If no Observation with code `105511-0` is present, then `ClinicalDocument.authorization.consent[code.code='59284-0']` is evaluated:  
-  - If `displayName = "yes"`, the Consent is set to "permit".  
-  - Otherwise, the Consent is set to "deny".
-If neither of the above values is available, the Consent defaults to "deny".</t>
+      <t xml:space="preserve"> CCDS, 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Case 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+The Consent value is first derived from the following path:
+`ClinicalDocument.component.structuredBody.component.section[code.code='29762-2'].entry.observation.entryRelationship.observation[code.code='105511-0']`
+If either of the following conditions is met:
+ value.code = 'LA33-6'
+ value.displayName = 'Permit'
+then the Consent is set to permit.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Case 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+If no consent is derived from Case 1, the Consent is evaluated from the following path:
+`ClinicalDocument.component.structuredBody.component.section[code.code='29762-2'].entry.observation.entryRelationship.observation`
+where:
+ templateId.root = '2.16.840.1.113883.10.20.22.4.86'
+ value.displayName = 'Permit'
+ value.xsi:type = 'CD'
+If such an Observation is present, the Consent is set to permit.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Case 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+If both Case 1 and Case 2 fail, the following path is evaluated:
+`ClinicalDocument.authorization.consent[code.code='59284-0']`
+If displayName = 'yes' or displayName = 'Permit', the Consent is set to permit.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Case 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+If none of the above conditions are satisfied, the Consent defaults to deny.</t>
     </r>
   </si>
   <si>
@@ -3478,7 +3530,8 @@
     <t>SHA-256 UUID generated using 
 1. Patient-MRN (the value set for 'identifier (MR) -&gt; value' of Patient Resource from Document.recordTarget.patientRole.id.extension)
 2. Value of the header variable 'X-TechBD-CIN'
-3. Content of first occurance of Document.author section</t>
+3. Content of first occurance of Document.author section
+4. Organization Name from Document.author.assignedAuthor.representedOrganization.name</t>
   </si>
   <si>
     <t>"id" : "8e4752d52cb9f94657401368f1c8e3cdb052624b10166a665e4c80cdabc62b3c",</t>
@@ -6007,6 +6060,22 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -6015,22 +6084,6 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -8414,7 +8467,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="105" customHeight="1" spans="1:7">
+    <row r="2" ht="380" customHeight="1" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
@@ -9037,7 +9090,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="4" ht="90" spans="1:6">
+    <row r="4" ht="135" spans="1:6">
       <c r="B4" t="s">
         <v>16</v>
       </c>

</xml_diff>